<commit_message>
feat: implement order detail page with status management and PI export functionality
</commit_message>
<xml_diff>
--- a/excel-template/PI-template.xlsx
+++ b/excel-template/PI-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\exportcrm\excel-template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EA7242-F286-40F7-BFA5-D7952BFE849F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC77D111-E184-4E64-A0E5-6CBB0952F14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
     <definedName name="Excel_BuiltIn_Print_Titles_1_1">#REF!</definedName>
     <definedName name="LISCO_LIMITED_UNIT_1603__16_F.__YEN_SHENG_CENTRE__64_HOI_YUEN_ROAD__KWUN_TONG__KOWLOON__HONG_KONG">#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">contract!$A$1:$G$57</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">PI!$A$1:$H$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">PI!$A$1:$H$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -689,7 +689,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -870,15 +870,6 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thin">
-        <color theme="2" tint="-0.24994659260841701"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
       <bottom style="medium">
         <color theme="2" tint="-9.9948118533890809E-2"/>
       </bottom>
@@ -911,7 +902,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="172">
+  <cellXfs count="166">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1209,29 +1200,8 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="20" fillId="0" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="20" fillId="0" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="43" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1249,86 +1219,107 @@
     <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="17" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="186" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="43" fontId="21" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="178" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="20" fillId="0" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="24" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="186" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="2" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1387,38 +1378,20 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="179" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="182" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="178" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1767,7 +1740,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:S38"/>
+  <dimension ref="A1:S35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="1" width="6.33203125" style="96" customWidth="1"/>
@@ -1792,21 +1765,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="55" customFormat="1" ht="66" customHeight="1">
-      <c r="A1" s="109"/>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="109"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="125" t="s">
+      <c r="A1" s="102"/>
+      <c r="B1" s="102"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="127" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="125"/>
-      <c r="H1" s="125"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
       <c r="N1" s="56"/>
       <c r="O1" s="56"/>
     </row>
     <row r="2" spans="1:19" ht="21.9" customHeight="1">
-      <c r="A2" s="110" t="s">
+      <c r="A2" s="103" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="95"/>
@@ -1816,16 +1789,16 @@
       <c r="F2" s="82" t="s">
         <v>80</v>
       </c>
-      <c r="G2" s="111" t="s">
+      <c r="G2" s="104" t="s">
         <v>86</v>
       </c>
-      <c r="H2" s="112"/>
+      <c r="H2" s="105"/>
     </row>
     <row r="3" spans="1:19" s="61" customFormat="1" ht="21.9" customHeight="1">
-      <c r="A3" s="113" t="s">
+      <c r="A3" s="106" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="114"/>
+      <c r="B3" s="107"/>
       <c r="C3" s="78"/>
       <c r="D3" s="77"/>
       <c r="E3" s="77"/>
@@ -1842,10 +1815,10 @@
       <c r="O3" s="62"/>
     </row>
     <row r="4" spans="1:19" s="61" customFormat="1" ht="21.9" customHeight="1">
-      <c r="A4" s="104" t="s">
+      <c r="A4" s="101" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="114"/>
+      <c r="B4" s="107"/>
       <c r="C4" s="78"/>
       <c r="D4" s="77"/>
       <c r="E4" s="77"/>
@@ -1866,18 +1839,18 @@
       <c r="Q4" s="67"/>
     </row>
     <row r="5" spans="1:19" s="61" customFormat="1" ht="21.75" customHeight="1" thickBot="1">
-      <c r="A5" s="115"/>
-      <c r="B5" s="116"/>
-      <c r="C5" s="117"/>
-      <c r="D5" s="118"/>
-      <c r="E5" s="118"/>
-      <c r="F5" s="119" t="s">
+      <c r="A5" s="108"/>
+      <c r="B5" s="109"/>
+      <c r="C5" s="110"/>
+      <c r="D5" s="111"/>
+      <c r="E5" s="111"/>
+      <c r="F5" s="112" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="119" t="s">
+      <c r="G5" s="112" t="s">
         <v>89</v>
       </c>
-      <c r="H5" s="119"/>
+      <c r="H5" s="112"/>
       <c r="J5" s="64"/>
       <c r="K5" s="65"/>
       <c r="L5" s="64"/>
@@ -1915,15 +1888,15 @@
       <c r="A7" s="76" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="126" t="s">
+      <c r="B7" s="128" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="126"/>
-      <c r="D7" s="126"/>
+      <c r="C7" s="128"/>
+      <c r="D7" s="128"/>
       <c r="E7" s="98"/>
-      <c r="F7" s="123"/>
-      <c r="G7" s="123"/>
-      <c r="H7" s="123"/>
+      <c r="F7" s="126"/>
+      <c r="G7" s="126"/>
+      <c r="H7" s="126"/>
       <c r="I7" s="67"/>
       <c r="J7" s="73"/>
       <c r="K7" s="67"/>
@@ -1939,15 +1912,15 @@
       <c r="A8" s="76" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="126" t="s">
+      <c r="B8" s="128" t="s">
         <v>79</v>
       </c>
-      <c r="C8" s="126"/>
-      <c r="D8" s="126"/>
+      <c r="C8" s="128"/>
+      <c r="D8" s="128"/>
       <c r="E8" s="98"/>
-      <c r="F8" s="123"/>
-      <c r="G8" s="123"/>
-      <c r="H8" s="123"/>
+      <c r="F8" s="126"/>
+      <c r="G8" s="126"/>
+      <c r="H8" s="126"/>
       <c r="I8" s="64"/>
       <c r="J8" s="64"/>
       <c r="K8" s="64"/>
@@ -1973,68 +1946,68 @@
       <c r="I9" s="77"/>
       <c r="J9" s="77"/>
       <c r="K9" s="77"/>
-      <c r="L9" s="122"/>
-      <c r="M9" s="122"/>
-      <c r="N9" s="122"/>
-      <c r="O9" s="122"/>
-      <c r="P9" s="122"/>
-      <c r="Q9" s="122"/>
-      <c r="R9" s="122"/>
-      <c r="S9" s="122"/>
+      <c r="L9" s="125"/>
+      <c r="M9" s="125"/>
+      <c r="N9" s="125"/>
+      <c r="O9" s="125"/>
+      <c r="P9" s="125"/>
+      <c r="Q9" s="125"/>
+      <c r="R9" s="125"/>
+      <c r="S9" s="125"/>
     </row>
     <row r="10" spans="1:19" s="79" customFormat="1" ht="26.25" customHeight="1">
-      <c r="A10" s="120" t="s">
+      <c r="A10" s="113" t="s">
         <v>3</v>
       </c>
       <c r="B10" s="130" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="130"/>
-      <c r="D10" s="120" t="s">
+      <c r="D10" s="113" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="120" t="s">
+      <c r="E10" s="113" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="120" t="s">
+      <c r="F10" s="113" t="s">
         <v>92</v>
       </c>
-      <c r="G10" s="120" t="s">
+      <c r="G10" s="113" t="s">
         <v>82</v>
       </c>
-      <c r="H10" s="120" t="s">
+      <c r="H10" s="113" t="s">
         <v>83</v>
       </c>
-      <c r="L10" s="122"/>
-      <c r="M10" s="122"/>
-      <c r="N10" s="122"/>
-      <c r="O10" s="122"/>
-      <c r="P10" s="122"/>
-      <c r="Q10" s="122"/>
-      <c r="R10" s="122"/>
-      <c r="S10" s="122"/>
+      <c r="L10" s="125"/>
+      <c r="M10" s="125"/>
+      <c r="N10" s="125"/>
+      <c r="O10" s="125"/>
+      <c r="P10" s="125"/>
+      <c r="Q10" s="125"/>
+      <c r="R10" s="125"/>
+      <c r="S10" s="125"/>
     </row>
     <row r="11" spans="1:19" s="78" customFormat="1" ht="28.5" customHeight="1">
-      <c r="A11" s="64">
+      <c r="A11" s="80">
         <v>1</v>
       </c>
-      <c r="B11" s="131" t="s">
+      <c r="B11" s="165" t="s">
         <v>90</v>
       </c>
-      <c r="C11" s="131"/>
-      <c r="D11" s="72" t="s">
+      <c r="C11" s="165"/>
+      <c r="D11" s="161" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="101">
+      <c r="E11" s="162">
         <v>250</v>
       </c>
-      <c r="F11" s="101" t="s">
+      <c r="F11" s="162" t="s">
         <v>93</v>
       </c>
-      <c r="G11" s="103">
+      <c r="G11" s="163">
         <v>14.3</v>
       </c>
-      <c r="H11" s="102">
+      <c r="H11" s="164">
         <v>3575</v>
       </c>
       <c r="K11" s="81"/>
@@ -2043,150 +2016,140 @@
       <c r="P11" s="82"/>
       <c r="Q11" s="82"/>
     </row>
-    <row r="12" spans="1:19" s="78" customFormat="1" ht="23.1" customHeight="1">
-      <c r="A12" s="64"/>
-      <c r="B12" s="127"/>
-      <c r="C12" s="127"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="101"/>
-      <c r="F12" s="101"/>
-      <c r="G12" s="103"/>
-      <c r="H12" s="102"/>
-      <c r="K12" s="81"/>
-      <c r="N12" s="77"/>
-      <c r="O12" s="77"/>
-      <c r="P12" s="82"/>
-      <c r="Q12" s="82"/>
-    </row>
-    <row r="13" spans="1:19" s="78" customFormat="1" ht="23.1" customHeight="1">
-      <c r="A13" s="64"/>
-      <c r="B13" s="127"/>
-      <c r="C13" s="127"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="72"/>
-      <c r="F13" s="101"/>
-      <c r="G13" s="102"/>
-      <c r="H13" s="102"/>
-      <c r="K13" s="81"/>
-      <c r="N13" s="77"/>
-      <c r="O13" s="77"/>
-      <c r="P13" s="82"/>
-      <c r="Q13" s="82"/>
-    </row>
-    <row r="14" spans="1:19" s="78" customFormat="1" ht="23.1" customHeight="1">
-      <c r="A14" s="105"/>
-      <c r="B14" s="128"/>
-      <c r="C14" s="128"/>
-      <c r="D14" s="106"/>
-      <c r="E14" s="106"/>
-      <c r="F14" s="107"/>
-      <c r="G14" s="108"/>
-      <c r="H14" s="108"/>
-      <c r="K14" s="81"/>
-      <c r="L14" s="77"/>
-      <c r="M14" s="77"/>
-      <c r="N14" s="77"/>
-      <c r="O14" s="77"/>
-      <c r="P14" s="77"/>
-      <c r="Q14" s="77"/>
-      <c r="R14" s="77"/>
-      <c r="S14" s="77"/>
-    </row>
-    <row r="15" spans="1:19" s="77" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A15" s="124" t="s">
+    <row r="12" spans="1:19" s="77" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A12" s="80" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="124"/>
-      <c r="C15" s="124"/>
-      <c r="D15" s="80"/>
-      <c r="E15" s="80"/>
-      <c r="F15" s="134" t="s">
+      <c r="B12" s="80"/>
+      <c r="C12" s="80"/>
+      <c r="D12" s="80"/>
+      <c r="E12" s="80"/>
+      <c r="F12" s="114" t="s">
         <v>14</v>
       </c>
-      <c r="G15" s="135" t="s">
+      <c r="G12" s="119" t="s">
         <v>94</v>
       </c>
-      <c r="H15" s="136">
-        <f>SUM(H11:H14)</f>
+      <c r="H12" s="120">
+        <f>SUM(H11:H11)</f>
         <v>3575</v>
       </c>
-      <c r="I15" s="83"/>
-    </row>
-    <row r="16" spans="1:19" s="77" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A16" s="124"/>
-      <c r="B16" s="124"/>
-      <c r="C16" s="124"/>
-      <c r="D16" s="80"/>
-      <c r="E16" s="80"/>
-      <c r="F16" s="134"/>
-      <c r="G16" s="135"/>
-      <c r="H16" s="136"/>
-    </row>
-    <row r="17" spans="1:19" s="77" customFormat="1" ht="30" customHeight="1">
-      <c r="A17" s="138" t="s">
+      <c r="I12" s="83"/>
+    </row>
+    <row r="13" spans="1:19" s="77" customFormat="1" ht="13.5" customHeight="1">
+      <c r="A13" s="80"/>
+      <c r="B13" s="80"/>
+      <c r="C13" s="80"/>
+      <c r="D13" s="80"/>
+      <c r="E13" s="80"/>
+      <c r="F13" s="114"/>
+      <c r="G13" s="119"/>
+      <c r="H13" s="120"/>
+    </row>
+    <row r="14" spans="1:19" s="77" customFormat="1" ht="30" customHeight="1">
+      <c r="A14" s="123" t="s">
         <v>84</v>
       </c>
-      <c r="B17" s="138"/>
-      <c r="C17" s="138"/>
-      <c r="D17" s="138"/>
-      <c r="E17" s="138"/>
-      <c r="F17" s="138"/>
-      <c r="G17" s="138"/>
-      <c r="H17" s="138"/>
+      <c r="B14" s="123"/>
+      <c r="C14" s="123"/>
+      <c r="D14" s="123"/>
+      <c r="E14" s="123"/>
+      <c r="F14" s="123"/>
+      <c r="G14" s="123"/>
+      <c r="H14" s="123"/>
+      <c r="K14" s="84"/>
+    </row>
+    <row r="15" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A15" s="121" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="121"/>
+      <c r="C15" s="121" t="s">
+        <v>95</v>
+      </c>
+      <c r="D15" s="121"/>
+      <c r="E15" s="121"/>
+      <c r="F15" s="121"/>
+      <c r="G15" s="121"/>
+      <c r="H15" s="85"/>
+      <c r="K15" s="84"/>
+    </row>
+    <row r="16" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A16" s="121" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="121"/>
+      <c r="C16" s="121" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="121"/>
+      <c r="E16" s="121"/>
+      <c r="F16" s="121"/>
+      <c r="G16" s="121"/>
+      <c r="H16" s="85"/>
+      <c r="K16" s="84"/>
+    </row>
+    <row r="17" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A17" s="121" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" s="121"/>
+      <c r="C17" s="121" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="121"/>
+      <c r="E17" s="121"/>
+      <c r="F17" s="121"/>
+      <c r="G17" s="121"/>
+      <c r="H17" s="85"/>
       <c r="K17" s="84"/>
     </row>
-    <row r="18" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="18" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A18" s="121" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="B18" s="121"/>
       <c r="C18" s="121" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D18" s="121"/>
       <c r="E18" s="121"/>
       <c r="F18" s="121"/>
       <c r="G18" s="121"/>
-      <c r="H18" s="85"/>
-      <c r="K18" s="84"/>
-    </row>
-    <row r="19" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+    </row>
+    <row r="19" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A19" s="121" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B19" s="121"/>
       <c r="C19" s="121" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="D19" s="121"/>
       <c r="E19" s="121"/>
       <c r="F19" s="121"/>
       <c r="G19" s="121"/>
-      <c r="H19" s="85"/>
-      <c r="K19" s="84"/>
-    </row>
-    <row r="20" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+    </row>
+    <row r="20" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A20" s="121" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B20" s="121"/>
       <c r="C20" s="121" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D20" s="121"/>
       <c r="E20" s="121"/>
       <c r="F20" s="121"/>
       <c r="G20" s="121"/>
-      <c r="H20" s="85"/>
-      <c r="K20" s="84"/>
     </row>
     <row r="21" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A21" s="121" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B21" s="121"/>
       <c r="C21" s="121" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="D21" s="121"/>
       <c r="E21" s="121"/>
@@ -2195,57 +2158,55 @@
     </row>
     <row r="22" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A22" s="121" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B22" s="121"/>
       <c r="C22" s="121" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D22" s="121"/>
       <c r="E22" s="121"/>
       <c r="F22" s="121"/>
       <c r="G22" s="121"/>
     </row>
-    <row r="23" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A23" s="121" t="s">
-        <v>103</v>
-      </c>
-      <c r="B23" s="121"/>
-      <c r="C23" s="121" t="s">
-        <v>107</v>
-      </c>
-      <c r="D23" s="121"/>
-      <c r="E23" s="121"/>
-      <c r="F23" s="121"/>
-      <c r="G23" s="121"/>
-    </row>
-    <row r="24" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A24" s="121" t="s">
-        <v>104</v>
-      </c>
-      <c r="B24" s="121"/>
-      <c r="C24" s="121" t="s">
-        <v>108</v>
-      </c>
-      <c r="D24" s="121"/>
-      <c r="E24" s="121"/>
-      <c r="F24" s="121"/>
-      <c r="G24" s="121"/>
-    </row>
-    <row r="25" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A25" s="121" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" s="121"/>
-      <c r="C25" s="121" t="s">
-        <v>109</v>
-      </c>
-      <c r="D25" s="121"/>
-      <c r="E25" s="121"/>
-      <c r="F25" s="121"/>
-      <c r="G25" s="121"/>
-    </row>
-    <row r="26" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="23" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A23" s="72"/>
+      <c r="B23" s="72"/>
+      <c r="C23" s="72"/>
+      <c r="D23" s="72"/>
+      <c r="E23" s="72"/>
+      <c r="F23" s="86"/>
+      <c r="G23" s="86"/>
+      <c r="H23" s="86"/>
+      <c r="K23" s="84"/>
+    </row>
+    <row r="24" spans="1:19" s="77" customFormat="1" ht="31.5" customHeight="1">
+      <c r="A24" s="122" t="s">
+        <v>110</v>
+      </c>
+      <c r="B24" s="122"/>
+      <c r="C24" s="122"/>
+      <c r="D24" s="122"/>
+      <c r="E24" s="122"/>
+      <c r="F24" s="122"/>
+      <c r="G24" s="122"/>
+      <c r="H24" s="122"/>
+      <c r="K24" s="84"/>
+    </row>
+    <row r="25" spans="1:19" s="70" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A25" s="124" t="s">
+        <v>112</v>
+      </c>
+      <c r="B25" s="124"/>
+      <c r="C25" s="124"/>
+      <c r="D25" s="124"/>
+      <c r="E25" s="124"/>
+      <c r="F25" s="87"/>
+      <c r="G25" s="87"/>
+      <c r="H25" s="87"/>
+      <c r="K25" s="88"/>
+    </row>
+    <row r="26" spans="1:19" s="77" customFormat="1" ht="27" customHeight="1">
       <c r="A26" s="72"/>
       <c r="B26" s="72"/>
       <c r="C26" s="72"/>
@@ -2255,208 +2216,166 @@
       <c r="G26" s="86"/>
       <c r="H26" s="86"/>
       <c r="K26" s="84"/>
-    </row>
-    <row r="27" spans="1:19" s="77" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A27" s="137" t="s">
-        <v>110</v>
-      </c>
-      <c r="B27" s="137"/>
-      <c r="C27" s="137"/>
-      <c r="D27" s="137"/>
-      <c r="E27" s="137"/>
-      <c r="F27" s="137"/>
-      <c r="G27" s="137"/>
-      <c r="H27" s="137"/>
-      <c r="K27" s="84"/>
-    </row>
-    <row r="28" spans="1:19" s="70" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A28" s="139" t="s">
-        <v>112</v>
-      </c>
-      <c r="B28" s="139"/>
-      <c r="C28" s="139"/>
-      <c r="D28" s="139"/>
-      <c r="E28" s="139"/>
-      <c r="F28" s="87"/>
-      <c r="G28" s="87"/>
-      <c r="H28" s="87"/>
-      <c r="K28" s="88"/>
-    </row>
-    <row r="29" spans="1:19" s="77" customFormat="1" ht="27" customHeight="1">
-      <c r="A29" s="72"/>
-      <c r="B29" s="72"/>
-      <c r="C29" s="72"/>
-      <c r="D29" s="72"/>
-      <c r="E29" s="72"/>
-      <c r="F29" s="86"/>
-      <c r="G29" s="86"/>
-      <c r="H29" s="86"/>
-      <c r="K29" s="84"/>
-      <c r="L29" s="89"/>
-      <c r="M29" s="89"/>
+      <c r="L26" s="89"/>
+      <c r="M26" s="89"/>
+      <c r="N26" s="90"/>
+      <c r="O26" s="90"/>
+      <c r="P26" s="89"/>
+      <c r="Q26" s="89"/>
+      <c r="R26" s="89"/>
+      <c r="S26" s="89"/>
+    </row>
+    <row r="27" spans="1:19" s="89" customFormat="1" ht="19.5" customHeight="1">
+      <c r="A27" s="117" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" s="117"/>
+      <c r="C27" s="117"/>
+      <c r="D27" s="117"/>
+      <c r="E27" s="117"/>
+      <c r="F27" s="117"/>
+      <c r="G27" s="117"/>
+      <c r="H27" s="117"/>
+      <c r="N27" s="90"/>
+      <c r="O27" s="90"/>
+    </row>
+    <row r="28" spans="1:19" s="89" customFormat="1" ht="53.25" customHeight="1">
+      <c r="A28" s="118" t="s">
+        <v>113</v>
+      </c>
+      <c r="B28" s="118"/>
+      <c r="C28" s="118"/>
+      <c r="D28" s="118"/>
+      <c r="E28" s="118"/>
+      <c r="F28" s="118"/>
+      <c r="G28" s="118"/>
+      <c r="H28" s="118"/>
+      <c r="N28" s="90"/>
+      <c r="O28" s="90"/>
+    </row>
+    <row r="29" spans="1:19" s="89" customFormat="1" ht="24" customHeight="1" thickBot="1">
+      <c r="A29" s="91"/>
+      <c r="B29" s="91"/>
+      <c r="C29" s="91"/>
+      <c r="D29" s="91"/>
+      <c r="E29" s="91"/>
+      <c r="F29" s="91"/>
+      <c r="G29" s="91"/>
+      <c r="H29" s="91"/>
       <c r="N29" s="90"/>
       <c r="O29" s="90"/>
-      <c r="P29" s="89"/>
-      <c r="Q29" s="89"/>
-      <c r="R29" s="89"/>
-      <c r="S29" s="89"/>
     </row>
     <row r="30" spans="1:19" s="89" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A30" s="132" t="s">
-        <v>111</v>
-      </c>
-      <c r="B30" s="132"/>
-      <c r="C30" s="132"/>
-      <c r="D30" s="132"/>
-      <c r="E30" s="132"/>
-      <c r="F30" s="132"/>
-      <c r="G30" s="132"/>
-      <c r="H30" s="132"/>
-      <c r="N30" s="90"/>
-      <c r="O30" s="90"/>
-    </row>
-    <row r="31" spans="1:19" s="89" customFormat="1" ht="53.25" customHeight="1">
-      <c r="A31" s="133" t="s">
-        <v>113</v>
-      </c>
-      <c r="B31" s="133"/>
-      <c r="C31" s="133"/>
-      <c r="D31" s="133"/>
-      <c r="E31" s="133"/>
-      <c r="F31" s="133"/>
-      <c r="G31" s="133"/>
-      <c r="H31" s="133"/>
-      <c r="N31" s="90"/>
-      <c r="O31" s="90"/>
-    </row>
-    <row r="32" spans="1:19" s="89" customFormat="1" ht="24" customHeight="1" thickBot="1">
-      <c r="A32" s="91"/>
-      <c r="B32" s="91"/>
-      <c r="C32" s="91"/>
-      <c r="D32" s="91"/>
-      <c r="E32" s="91"/>
-      <c r="F32" s="91"/>
-      <c r="G32" s="91"/>
-      <c r="H32" s="91"/>
-      <c r="N32" s="90"/>
-      <c r="O32" s="90"/>
-    </row>
-    <row r="33" spans="1:19" s="89" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A33" s="141" t="s">
+      <c r="A30" s="116" t="s">
         <v>18</v>
       </c>
-      <c r="B33" s="141"/>
-      <c r="C33" s="141"/>
-      <c r="D33" s="141"/>
-      <c r="E33" s="141" t="s">
+      <c r="B30" s="116"/>
+      <c r="C30" s="116"/>
+      <c r="D30" s="116"/>
+      <c r="E30" s="116" t="s">
         <v>19</v>
       </c>
-      <c r="F33" s="141"/>
-      <c r="G33" s="141"/>
-      <c r="H33" s="141"/>
-      <c r="L33" s="57"/>
-      <c r="M33" s="57"/>
-      <c r="N33" s="60"/>
-      <c r="O33" s="60"/>
-      <c r="P33" s="57"/>
-      <c r="Q33" s="57"/>
-      <c r="R33" s="57"/>
-      <c r="S33" s="57"/>
-    </row>
-    <row r="34" spans="1:19">
-      <c r="A34" s="93" t="s">
+      <c r="F30" s="116"/>
+      <c r="G30" s="116"/>
+      <c r="H30" s="116"/>
+      <c r="L30" s="57"/>
+      <c r="M30" s="57"/>
+      <c r="N30" s="60"/>
+      <c r="O30" s="60"/>
+      <c r="P30" s="57"/>
+      <c r="Q30" s="57"/>
+      <c r="R30" s="57"/>
+      <c r="S30" s="57"/>
+    </row>
+    <row r="31" spans="1:19">
+      <c r="A31" s="93" t="s">
         <v>20</v>
       </c>
-      <c r="C34" s="94"/>
-      <c r="D34" s="95"/>
-      <c r="E34" s="140" t="s">
+      <c r="C31" s="94"/>
+      <c r="D31" s="95"/>
+      <c r="E31" s="115" t="s">
         <v>21</v>
       </c>
-      <c r="F34" s="140"/>
-      <c r="G34" s="140"/>
-      <c r="H34" s="140"/>
-    </row>
-    <row r="35" spans="1:19">
-      <c r="A35" s="140" t="s">
+      <c r="F31" s="115"/>
+      <c r="G31" s="115"/>
+      <c r="H31" s="115"/>
+    </row>
+    <row r="32" spans="1:19">
+      <c r="A32" s="115" t="s">
         <v>22</v>
       </c>
-      <c r="B35" s="140"/>
-      <c r="C35" s="140"/>
-      <c r="D35" s="140"/>
-      <c r="E35" s="140" t="s">
+      <c r="B32" s="115"/>
+      <c r="C32" s="115"/>
+      <c r="D32" s="115"/>
+      <c r="E32" s="115" t="s">
         <v>23</v>
       </c>
-      <c r="F35" s="140"/>
-      <c r="G35" s="140"/>
-      <c r="H35" s="140"/>
-    </row>
-    <row r="36" spans="1:19">
-      <c r="A36" s="140" t="s">
+      <c r="F32" s="115"/>
+      <c r="G32" s="115"/>
+      <c r="H32" s="115"/>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="115" t="s">
         <v>24</v>
       </c>
-      <c r="B36" s="140"/>
-      <c r="C36" s="140"/>
-      <c r="D36" s="140"/>
-      <c r="E36" s="140" t="s">
+      <c r="B33" s="115"/>
+      <c r="C33" s="115"/>
+      <c r="D33" s="115"/>
+      <c r="E33" s="115" t="s">
         <v>25</v>
       </c>
-      <c r="F36" s="140"/>
-      <c r="G36" s="140"/>
-      <c r="H36" s="140"/>
-    </row>
-    <row r="37" spans="1:19">
-      <c r="A37" s="55"/>
-      <c r="F37" s="55"/>
-      <c r="H37" s="92"/>
-    </row>
-    <row r="38" spans="1:19">
-      <c r="A38" s="63"/>
+      <c r="F33" s="115"/>
+      <c r="G33" s="115"/>
+      <c r="H33" s="115"/>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="55"/>
+      <c r="F34" s="55"/>
+      <c r="H34" s="92"/>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="63"/>
     </row>
   </sheetData>
-  <mergeCells count="43">
-    <mergeCell ref="E36:H36"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A36:D36"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="E33:H33"/>
-    <mergeCell ref="E34:H34"/>
-    <mergeCell ref="E35:H35"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="A18:B18"/>
+  <mergeCells count="38">
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C22:G22"/>
     <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:G19"/>
     <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C20:G20"/>
     <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="C18:G18"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="C20:G20"/>
     <mergeCell ref="C21:G21"/>
-    <mergeCell ref="A28:E28"/>
     <mergeCell ref="L9:S10"/>
     <mergeCell ref="F7:H8"/>
-    <mergeCell ref="A15:C16"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:G25"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="E33:H33"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="E30:H30"/>
+    <mergeCell ref="E31:H31"/>
+    <mergeCell ref="E32:H32"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <hyperlinks>
@@ -2494,15 +2413,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A1" s="167" t="s">
+      <c r="A1" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="167"/>
-      <c r="C1" s="167"/>
-      <c r="D1" s="167"/>
-      <c r="E1" s="167"/>
-      <c r="F1" s="167"/>
-      <c r="G1" s="167"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
       <c r="M1" s="45"/>
       <c r="N1" s="45"/>
     </row>
@@ -2540,14 +2459,14 @@
     </row>
     <row r="5" spans="1:15" s="2" customFormat="1" ht="33" customHeight="1">
       <c r="A5" s="17"/>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="132" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="168"/>
-      <c r="D5" s="168"/>
-      <c r="E5" s="168"/>
-      <c r="F5" s="168"/>
-      <c r="G5" s="168"/>
+      <c r="C5" s="132"/>
+      <c r="D5" s="132"/>
+      <c r="E5" s="132"/>
+      <c r="F5" s="132"/>
+      <c r="G5" s="132"/>
       <c r="H5" s="18"/>
       <c r="M5" s="46"/>
       <c r="N5" s="46"/>
@@ -2567,27 +2486,27 @@
       <c r="A7" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="169" t="s">
+      <c r="B7" s="133" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="169"/>
-      <c r="D7" s="169"/>
-      <c r="E7" s="169"/>
-      <c r="F7" s="169"/>
+      <c r="C7" s="133"/>
+      <c r="D7" s="133"/>
+      <c r="E7" s="133"/>
+      <c r="F7" s="133"/>
       <c r="G7" s="20"/>
       <c r="M7" s="46"/>
       <c r="N7" s="46"/>
     </row>
     <row r="8" spans="1:15" s="2" customFormat="1" ht="54" customHeight="1">
       <c r="A8" s="17"/>
-      <c r="B8" s="170" t="s">
+      <c r="B8" s="134" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="170"/>
-      <c r="D8" s="170"/>
-      <c r="E8" s="170"/>
-      <c r="F8" s="170"/>
-      <c r="G8" s="170"/>
+      <c r="C8" s="134"/>
+      <c r="D8" s="134"/>
+      <c r="E8" s="134"/>
+      <c r="F8" s="134"/>
+      <c r="G8" s="134"/>
       <c r="M8" s="46"/>
       <c r="N8" s="46"/>
     </row>
@@ -2603,28 +2522,28 @@
       <c r="N9" s="46"/>
     </row>
     <row r="10" spans="1:15" s="3" customFormat="1" ht="49.5" customHeight="1">
-      <c r="A10" s="171" t="s">
+      <c r="A10" s="135" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="171"/>
-      <c r="C10" s="171"/>
-      <c r="D10" s="171"/>
-      <c r="E10" s="171"/>
-      <c r="F10" s="171"/>
-      <c r="G10" s="171"/>
+      <c r="B10" s="135"/>
+      <c r="C10" s="135"/>
+      <c r="D10" s="135"/>
+      <c r="E10" s="135"/>
+      <c r="F10" s="135"/>
+      <c r="G10" s="135"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
     </row>
     <row r="11" spans="1:15" s="3" customFormat="1" ht="27" customHeight="1">
-      <c r="A11" s="164" t="s">
+      <c r="A11" s="136" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="164"/>
-      <c r="C11" s="164"/>
-      <c r="D11" s="164"/>
-      <c r="E11" s="164"/>
-      <c r="F11" s="164"/>
-      <c r="G11" s="164"/>
+      <c r="B11" s="136"/>
+      <c r="C11" s="136"/>
+      <c r="D11" s="136"/>
+      <c r="E11" s="136"/>
+      <c r="F11" s="136"/>
+      <c r="G11" s="136"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
     </row>
@@ -2632,10 +2551,10 @@
       <c r="A12" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="165" t="s">
+      <c r="B12" s="137" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="166"/>
+      <c r="C12" s="138"/>
       <c r="D12" s="23" t="s">
         <v>5</v>
       </c>
@@ -2657,10 +2576,10 @@
       <c r="A13" s="25">
         <v>1</v>
       </c>
-      <c r="B13" s="161">
+      <c r="B13" s="139">
         <v>50655</v>
       </c>
-      <c r="C13" s="162"/>
+      <c r="C13" s="140"/>
       <c r="D13" s="26" t="s">
         <v>7</v>
       </c>
@@ -2683,10 +2602,10 @@
       <c r="A14" s="25">
         <v>2</v>
       </c>
-      <c r="B14" s="161">
+      <c r="B14" s="139">
         <v>50755</v>
       </c>
-      <c r="C14" s="162"/>
+      <c r="C14" s="140"/>
       <c r="D14" s="26" t="s">
         <v>8</v>
       </c>
@@ -2709,10 +2628,10 @@
       <c r="A15" s="25">
         <v>3</v>
       </c>
-      <c r="B15" s="161">
+      <c r="B15" s="139">
         <v>50665</v>
       </c>
-      <c r="C15" s="162"/>
+      <c r="C15" s="140"/>
       <c r="D15" s="26" t="s">
         <v>9</v>
       </c>
@@ -2735,10 +2654,10 @@
       <c r="A16" s="25">
         <v>4</v>
       </c>
-      <c r="B16" s="161">
+      <c r="B16" s="139">
         <v>50765</v>
       </c>
-      <c r="C16" s="162"/>
+      <c r="C16" s="140"/>
       <c r="D16" s="26" t="s">
         <v>10</v>
       </c>
@@ -2761,10 +2680,10 @@
       <c r="A17" s="25">
         <v>5</v>
       </c>
-      <c r="B17" s="161">
+      <c r="B17" s="139">
         <v>50720</v>
       </c>
-      <c r="C17" s="162"/>
+      <c r="C17" s="140"/>
       <c r="D17" s="26" t="s">
         <v>11</v>
       </c>
@@ -2787,10 +2706,10 @@
       <c r="A18" s="30">
         <v>6</v>
       </c>
-      <c r="B18" s="161">
+      <c r="B18" s="139">
         <v>50730</v>
       </c>
-      <c r="C18" s="162"/>
+      <c r="C18" s="140"/>
       <c r="D18" s="31" t="s">
         <v>12</v>
       </c>
@@ -2837,15 +2756,15 @@
       <c r="G20" s="148"/>
     </row>
     <row r="21" spans="1:15" s="4" customFormat="1" ht="30" hidden="1" customHeight="1">
-      <c r="A21" s="163" t="s">
+      <c r="A21" s="141" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="163"/>
-      <c r="C21" s="163"/>
-      <c r="D21" s="163"/>
-      <c r="E21" s="163"/>
-      <c r="F21" s="163"/>
-      <c r="G21" s="163"/>
+      <c r="B21" s="141"/>
+      <c r="C21" s="141"/>
+      <c r="D21" s="141"/>
+      <c r="E21" s="141"/>
+      <c r="F21" s="141"/>
+      <c r="G21" s="141"/>
       <c r="J21" s="52"/>
     </row>
     <row r="22" spans="1:15" s="4" customFormat="1" ht="30" customHeight="1">
@@ -3223,21 +3142,6 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A50:G50"/>
     <mergeCell ref="E19:E20"/>
     <mergeCell ref="F19:F20"/>
@@ -3254,6 +3158,21 @@
     <mergeCell ref="A37:G37"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A41:G41"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="A10:G10"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>

<commit_message>
feat: implement dashboard components, internationalization support, and core service modules for orders and payments
</commit_message>
<xml_diff>
--- a/excel-template/PI-template.xlsx
+++ b/excel-template/PI-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\exportcrm\excel-template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC77D111-E184-4E64-A0E5-6CBB0952F14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2818FCBC-5192-4563-8666-69B64136EFF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="114">
   <si>
     <t>Chongqing Alustars International Co.,Ltd.</t>
   </si>
@@ -373,16 +373,6 @@
     <phoneticPr fontId="15" type="noConversion"/>
   </si>
   <si>
-    <t>0080-2062-0843
-Iss.6-1/2</t>
-    <phoneticPr fontId="15" type="noConversion"/>
-  </si>
-  <si>
-    <t>Pilot Light Torch Tube
-HS code: 7326909890</t>
-    <phoneticPr fontId="15" type="noConversion"/>
-  </si>
-  <si>
     <t>Unit</t>
     <phoneticPr fontId="15" type="noConversion"/>
   </si>
@@ -469,6 +459,14 @@
   <si>
     <t xml:space="preserve">    Carlos Feliu
     VP of Business Development                                                      (Company Seal)</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pilot Light Torch Tube</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>0080-2062-0843</t>
     <phoneticPr fontId="15" type="noConversion"/>
   </si>
 </sst>
@@ -689,7 +687,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -884,6 +882,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color theme="2" tint="-9.9948118533890809E-2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -902,7 +909,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="166">
+  <cellXfs count="168">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1207,87 +1214,105 @@
     <xf numFmtId="43" fontId="18" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="179" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="182" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="186" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="43" fontId="21" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="24" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="17" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="186" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="43" fontId="21" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="24" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1378,20 +1403,8 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="179" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="182" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="178" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="43" fontId="17" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1770,11 +1783,11 @@
       <c r="C1" s="102"/>
       <c r="D1" s="102"/>
       <c r="E1" s="102"/>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="130" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
+      <c r="G1" s="130"/>
+      <c r="H1" s="130"/>
       <c r="N1" s="56"/>
       <c r="O1" s="56"/>
     </row>
@@ -1789,28 +1802,26 @@
       <c r="F2" s="82" t="s">
         <v>80</v>
       </c>
-      <c r="G2" s="104" t="s">
+      <c r="G2" s="134" t="s">
         <v>86</v>
       </c>
-      <c r="H2" s="105"/>
+      <c r="H2" s="134"/>
     </row>
     <row r="3" spans="1:19" s="61" customFormat="1" ht="21.9" customHeight="1">
-      <c r="A3" s="106" t="s">
+      <c r="A3" s="104" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="107"/>
+      <c r="B3" s="105"/>
       <c r="C3" s="78"/>
       <c r="D3" s="77"/>
       <c r="E3" s="77"/>
       <c r="F3" s="82" t="s">
         <v>69</v>
       </c>
-      <c r="G3" s="82" t="s">
+      <c r="G3" s="135" t="s">
         <v>87</v>
       </c>
-      <c r="H3" s="82" t="s">
-        <v>68</v>
-      </c>
+      <c r="H3" s="135"/>
       <c r="N3" s="62"/>
       <c r="O3" s="62"/>
     </row>
@@ -1818,17 +1829,17 @@
       <c r="A4" s="101" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="107"/>
+      <c r="B4" s="105"/>
       <c r="C4" s="78"/>
       <c r="D4" s="77"/>
       <c r="E4" s="77"/>
       <c r="F4" s="82" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="82" t="s">
+      <c r="G4" s="135" t="s">
         <v>88</v>
       </c>
-      <c r="H4" s="82"/>
+      <c r="H4" s="135"/>
       <c r="J4" s="64"/>
       <c r="K4" s="65"/>
       <c r="L4" s="64"/>
@@ -1839,18 +1850,18 @@
       <c r="Q4" s="67"/>
     </row>
     <row r="5" spans="1:19" s="61" customFormat="1" ht="21.75" customHeight="1" thickBot="1">
-      <c r="A5" s="108"/>
-      <c r="B5" s="109"/>
-      <c r="C5" s="110"/>
-      <c r="D5" s="111"/>
-      <c r="E5" s="111"/>
-      <c r="F5" s="112" t="s">
+      <c r="A5" s="106"/>
+      <c r="B5" s="107"/>
+      <c r="C5" s="108"/>
+      <c r="D5" s="109"/>
+      <c r="E5" s="109"/>
+      <c r="F5" s="110" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="112" t="s">
+      <c r="G5" s="136" t="s">
         <v>89</v>
       </c>
-      <c r="H5" s="112"/>
+      <c r="H5" s="136"/>
       <c r="J5" s="64"/>
       <c r="K5" s="65"/>
       <c r="L5" s="64"/>
@@ -1864,11 +1875,11 @@
       <c r="A6" s="97" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="66" t="s">
+      <c r="B6" s="167" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
+      <c r="C6" s="167"/>
+      <c r="D6" s="167"/>
       <c r="E6" s="68"/>
       <c r="F6" s="99"/>
       <c r="G6" s="100"/>
@@ -1888,15 +1899,15 @@
       <c r="A7" s="76" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="128" t="s">
+      <c r="B7" s="131" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="128"/>
-      <c r="D7" s="128"/>
+      <c r="C7" s="131"/>
+      <c r="D7" s="131"/>
       <c r="E7" s="98"/>
-      <c r="F7" s="126"/>
-      <c r="G7" s="126"/>
-      <c r="H7" s="126"/>
+      <c r="F7" s="129"/>
+      <c r="G7" s="129"/>
+      <c r="H7" s="129"/>
       <c r="I7" s="67"/>
       <c r="J7" s="73"/>
       <c r="K7" s="67"/>
@@ -1912,15 +1923,15 @@
       <c r="A8" s="76" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="128" t="s">
+      <c r="B8" s="131" t="s">
         <v>79</v>
       </c>
-      <c r="C8" s="128"/>
-      <c r="D8" s="128"/>
+      <c r="C8" s="131"/>
+      <c r="D8" s="131"/>
       <c r="E8" s="98"/>
-      <c r="F8" s="126"/>
-      <c r="G8" s="126"/>
-      <c r="H8" s="126"/>
+      <c r="F8" s="129"/>
+      <c r="G8" s="129"/>
+      <c r="H8" s="129"/>
       <c r="I8" s="64"/>
       <c r="J8" s="64"/>
       <c r="K8" s="64"/>
@@ -1933,81 +1944,81 @@
       <c r="R8" s="73"/>
     </row>
     <row r="9" spans="1:19" s="78" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A9" s="129" t="s">
+      <c r="A9" s="132" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="129"/>
-      <c r="C9" s="129"/>
-      <c r="D9" s="129"/>
-      <c r="E9" s="129"/>
-      <c r="F9" s="129"/>
-      <c r="G9" s="129"/>
-      <c r="H9" s="129"/>
+      <c r="B9" s="132"/>
+      <c r="C9" s="132"/>
+      <c r="D9" s="132"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="132"/>
+      <c r="G9" s="132"/>
+      <c r="H9" s="132"/>
       <c r="I9" s="77"/>
       <c r="J9" s="77"/>
       <c r="K9" s="77"/>
-      <c r="L9" s="125"/>
-      <c r="M9" s="125"/>
-      <c r="N9" s="125"/>
-      <c r="O9" s="125"/>
-      <c r="P9" s="125"/>
-      <c r="Q9" s="125"/>
-      <c r="R9" s="125"/>
-      <c r="S9" s="125"/>
+      <c r="L9" s="128"/>
+      <c r="M9" s="128"/>
+      <c r="N9" s="128"/>
+      <c r="O9" s="128"/>
+      <c r="P9" s="128"/>
+      <c r="Q9" s="128"/>
+      <c r="R9" s="128"/>
+      <c r="S9" s="128"/>
     </row>
     <row r="10" spans="1:19" s="79" customFormat="1" ht="26.25" customHeight="1">
-      <c r="A10" s="113" t="s">
+      <c r="A10" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="130" t="s">
+      <c r="B10" s="133" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="130"/>
-      <c r="D10" s="113" t="s">
+      <c r="C10" s="133"/>
+      <c r="D10" s="111" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="113" t="s">
+      <c r="E10" s="111" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="113" t="s">
-        <v>92</v>
-      </c>
-      <c r="G10" s="113" t="s">
+      <c r="F10" s="111" t="s">
+        <v>90</v>
+      </c>
+      <c r="G10" s="111" t="s">
         <v>82</v>
       </c>
-      <c r="H10" s="113" t="s">
+      <c r="H10" s="111" t="s">
         <v>83</v>
       </c>
-      <c r="L10" s="125"/>
-      <c r="M10" s="125"/>
-      <c r="N10" s="125"/>
-      <c r="O10" s="125"/>
-      <c r="P10" s="125"/>
-      <c r="Q10" s="125"/>
-      <c r="R10" s="125"/>
-      <c r="S10" s="125"/>
-    </row>
-    <row r="11" spans="1:19" s="78" customFormat="1" ht="28.5" customHeight="1">
+      <c r="L10" s="128"/>
+      <c r="M10" s="128"/>
+      <c r="N10" s="128"/>
+      <c r="O10" s="128"/>
+      <c r="P10" s="128"/>
+      <c r="Q10" s="128"/>
+      <c r="R10" s="128"/>
+      <c r="S10" s="128"/>
+    </row>
+    <row r="11" spans="1:19" s="78" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A11" s="80">
         <v>1</v>
       </c>
-      <c r="B11" s="165" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" s="165"/>
-      <c r="D11" s="161" t="s">
+      <c r="B11" s="119" t="s">
+        <v>113</v>
+      </c>
+      <c r="C11" s="119"/>
+      <c r="D11" s="113" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" s="114">
+        <v>250</v>
+      </c>
+      <c r="F11" s="114" t="s">
         <v>91</v>
       </c>
-      <c r="E11" s="162">
-        <v>250</v>
-      </c>
-      <c r="F11" s="162" t="s">
-        <v>93</v>
-      </c>
-      <c r="G11" s="163">
+      <c r="G11" s="115">
         <v>14.3</v>
       </c>
-      <c r="H11" s="164">
+      <c r="H11" s="116">
         <v>3575</v>
       </c>
       <c r="K11" s="81"/>
@@ -2024,13 +2035,13 @@
       <c r="C12" s="80"/>
       <c r="D12" s="80"/>
       <c r="E12" s="80"/>
-      <c r="F12" s="114" t="s">
+      <c r="F12" s="112" t="s">
         <v>14</v>
       </c>
-      <c r="G12" s="119" t="s">
-        <v>94</v>
-      </c>
-      <c r="H12" s="120">
+      <c r="G12" s="122" t="s">
+        <v>92</v>
+      </c>
+      <c r="H12" s="123">
         <f>SUM(H11:H11)</f>
         <v>3575</v>
       </c>
@@ -2042,132 +2053,132 @@
       <c r="C13" s="80"/>
       <c r="D13" s="80"/>
       <c r="E13" s="80"/>
-      <c r="F13" s="114"/>
-      <c r="G13" s="119"/>
-      <c r="H13" s="120"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="122"/>
+      <c r="H13" s="123"/>
     </row>
     <row r="14" spans="1:19" s="77" customFormat="1" ht="30" customHeight="1">
-      <c r="A14" s="123" t="s">
+      <c r="A14" s="126" t="s">
         <v>84</v>
       </c>
-      <c r="B14" s="123"/>
-      <c r="C14" s="123"/>
-      <c r="D14" s="123"/>
-      <c r="E14" s="123"/>
-      <c r="F14" s="123"/>
-      <c r="G14" s="123"/>
-      <c r="H14" s="123"/>
+      <c r="B14" s="126"/>
+      <c r="C14" s="126"/>
+      <c r="D14" s="126"/>
+      <c r="E14" s="126"/>
+      <c r="F14" s="126"/>
+      <c r="G14" s="126"/>
+      <c r="H14" s="126"/>
       <c r="K14" s="84"/>
     </row>
     <row r="15" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A15" s="121" t="s">
+      <c r="A15" s="124" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="121"/>
-      <c r="C15" s="121" t="s">
-        <v>95</v>
-      </c>
-      <c r="D15" s="121"/>
-      <c r="E15" s="121"/>
-      <c r="F15" s="121"/>
-      <c r="G15" s="121"/>
+      <c r="B15" s="124"/>
+      <c r="C15" s="124" t="s">
+        <v>93</v>
+      </c>
+      <c r="D15" s="124"/>
+      <c r="E15" s="124"/>
+      <c r="F15" s="124"/>
+      <c r="G15" s="124"/>
       <c r="H15" s="85"/>
       <c r="K15" s="84"/>
     </row>
     <row r="16" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A16" s="121" t="s">
-        <v>96</v>
-      </c>
-      <c r="B16" s="121"/>
-      <c r="C16" s="121" t="s">
-        <v>97</v>
-      </c>
-      <c r="D16" s="121"/>
-      <c r="E16" s="121"/>
-      <c r="F16" s="121"/>
-      <c r="G16" s="121"/>
+      <c r="A16" s="124" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="124"/>
+      <c r="C16" s="124" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="124"/>
+      <c r="E16" s="124"/>
+      <c r="F16" s="124"/>
+      <c r="G16" s="124"/>
       <c r="H16" s="85"/>
       <c r="K16" s="84"/>
     </row>
     <row r="17" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A17" s="121" t="s">
-        <v>98</v>
-      </c>
-      <c r="B17" s="121"/>
-      <c r="C17" s="121" t="s">
-        <v>101</v>
-      </c>
-      <c r="D17" s="121"/>
-      <c r="E17" s="121"/>
-      <c r="F17" s="121"/>
-      <c r="G17" s="121"/>
+      <c r="A17" s="124" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" s="124"/>
+      <c r="C17" s="124" t="s">
+        <v>99</v>
+      </c>
+      <c r="D17" s="124"/>
+      <c r="E17" s="124"/>
+      <c r="F17" s="124"/>
+      <c r="G17" s="124"/>
       <c r="H17" s="85"/>
       <c r="K17" s="84"/>
     </row>
     <row r="18" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A18" s="121" t="s">
+      <c r="A18" s="124" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" s="124"/>
+      <c r="C18" s="124" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="124"/>
+      <c r="E18" s="124"/>
+      <c r="F18" s="124"/>
+      <c r="G18" s="124"/>
+    </row>
+    <row r="19" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A19" s="124" t="s">
         <v>100</v>
       </c>
-      <c r="B18" s="121"/>
-      <c r="C18" s="121" t="s">
-        <v>99</v>
-      </c>
-      <c r="D18" s="121"/>
-      <c r="E18" s="121"/>
-      <c r="F18" s="121"/>
-      <c r="G18" s="121"/>
-    </row>
-    <row r="19" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A19" s="121" t="s">
+      <c r="B19" s="124"/>
+      <c r="C19" s="124" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="124"/>
+      <c r="E19" s="124"/>
+      <c r="F19" s="124"/>
+      <c r="G19" s="124"/>
+    </row>
+    <row r="20" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A20" s="124" t="s">
+        <v>101</v>
+      </c>
+      <c r="B20" s="124"/>
+      <c r="C20" s="124" t="s">
+        <v>105</v>
+      </c>
+      <c r="D20" s="124"/>
+      <c r="E20" s="124"/>
+      <c r="F20" s="124"/>
+      <c r="G20" s="124"/>
+    </row>
+    <row r="21" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A21" s="124" t="s">
         <v>102</v>
       </c>
-      <c r="B19" s="121"/>
-      <c r="C19" s="121" t="s">
+      <c r="B21" s="124"/>
+      <c r="C21" s="124" t="s">
         <v>106</v>
       </c>
-      <c r="D19" s="121"/>
-      <c r="E19" s="121"/>
-      <c r="F19" s="121"/>
-      <c r="G19" s="121"/>
-    </row>
-    <row r="20" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A20" s="121" t="s">
+      <c r="D21" s="124"/>
+      <c r="E21" s="124"/>
+      <c r="F21" s="124"/>
+      <c r="G21" s="124"/>
+    </row>
+    <row r="22" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A22" s="124" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="121"/>
-      <c r="C20" s="121" t="s">
+      <c r="B22" s="124"/>
+      <c r="C22" s="124" t="s">
         <v>107</v>
       </c>
-      <c r="D20" s="121"/>
-      <c r="E20" s="121"/>
-      <c r="F20" s="121"/>
-      <c r="G20" s="121"/>
-    </row>
-    <row r="21" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A21" s="121" t="s">
-        <v>104</v>
-      </c>
-      <c r="B21" s="121"/>
-      <c r="C21" s="121" t="s">
-        <v>108</v>
-      </c>
-      <c r="D21" s="121"/>
-      <c r="E21" s="121"/>
-      <c r="F21" s="121"/>
-      <c r="G21" s="121"/>
-    </row>
-    <row r="22" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A22" s="121" t="s">
-        <v>105</v>
-      </c>
-      <c r="B22" s="121"/>
-      <c r="C22" s="121" t="s">
-        <v>109</v>
-      </c>
-      <c r="D22" s="121"/>
-      <c r="E22" s="121"/>
-      <c r="F22" s="121"/>
-      <c r="G22" s="121"/>
+      <c r="D22" s="124"/>
+      <c r="E22" s="124"/>
+      <c r="F22" s="124"/>
+      <c r="G22" s="124"/>
     </row>
     <row r="23" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
       <c r="A23" s="72"/>
@@ -2181,26 +2192,26 @@
       <c r="K23" s="84"/>
     </row>
     <row r="24" spans="1:19" s="77" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A24" s="122" t="s">
+      <c r="A24" s="125" t="s">
+        <v>108</v>
+      </c>
+      <c r="B24" s="125"/>
+      <c r="C24" s="125"/>
+      <c r="D24" s="125"/>
+      <c r="E24" s="125"/>
+      <c r="F24" s="125"/>
+      <c r="G24" s="125"/>
+      <c r="H24" s="125"/>
+      <c r="K24" s="84"/>
+    </row>
+    <row r="25" spans="1:19" s="70" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="A25" s="127" t="s">
         <v>110</v>
       </c>
-      <c r="B24" s="122"/>
-      <c r="C24" s="122"/>
-      <c r="D24" s="122"/>
-      <c r="E24" s="122"/>
-      <c r="F24" s="122"/>
-      <c r="G24" s="122"/>
-      <c r="H24" s="122"/>
-      <c r="K24" s="84"/>
-    </row>
-    <row r="25" spans="1:19" s="70" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A25" s="124" t="s">
-        <v>112</v>
-      </c>
-      <c r="B25" s="124"/>
-      <c r="C25" s="124"/>
-      <c r="D25" s="124"/>
-      <c r="E25" s="124"/>
+      <c r="B25" s="127"/>
+      <c r="C25" s="127"/>
+      <c r="D25" s="127"/>
+      <c r="E25" s="127"/>
       <c r="F25" s="87"/>
       <c r="G25" s="87"/>
       <c r="H25" s="87"/>
@@ -2226,30 +2237,30 @@
       <c r="S26" s="89"/>
     </row>
     <row r="27" spans="1:19" s="89" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A27" s="117" t="s">
-        <v>111</v>
-      </c>
-      <c r="B27" s="117"/>
-      <c r="C27" s="117"/>
-      <c r="D27" s="117"/>
-      <c r="E27" s="117"/>
-      <c r="F27" s="117"/>
-      <c r="G27" s="117"/>
-      <c r="H27" s="117"/>
+      <c r="A27" s="120" t="s">
+        <v>109</v>
+      </c>
+      <c r="B27" s="120"/>
+      <c r="C27" s="120"/>
+      <c r="D27" s="120"/>
+      <c r="E27" s="120"/>
+      <c r="F27" s="120"/>
+      <c r="G27" s="120"/>
+      <c r="H27" s="120"/>
       <c r="N27" s="90"/>
       <c r="O27" s="90"/>
     </row>
     <row r="28" spans="1:19" s="89" customFormat="1" ht="53.25" customHeight="1">
-      <c r="A28" s="118" t="s">
-        <v>113</v>
-      </c>
-      <c r="B28" s="118"/>
-      <c r="C28" s="118"/>
-      <c r="D28" s="118"/>
-      <c r="E28" s="118"/>
-      <c r="F28" s="118"/>
-      <c r="G28" s="118"/>
-      <c r="H28" s="118"/>
+      <c r="A28" s="121" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" s="121"/>
+      <c r="C28" s="121"/>
+      <c r="D28" s="121"/>
+      <c r="E28" s="121"/>
+      <c r="F28" s="121"/>
+      <c r="G28" s="121"/>
+      <c r="H28" s="121"/>
       <c r="N28" s="90"/>
       <c r="O28" s="90"/>
     </row>
@@ -2266,18 +2277,18 @@
       <c r="O29" s="90"/>
     </row>
     <row r="30" spans="1:19" s="89" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A30" s="116" t="s">
+      <c r="A30" s="118" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="116"/>
-      <c r="C30" s="116"/>
-      <c r="D30" s="116"/>
-      <c r="E30" s="116" t="s">
+      <c r="B30" s="118"/>
+      <c r="C30" s="118"/>
+      <c r="D30" s="118"/>
+      <c r="E30" s="118" t="s">
         <v>19</v>
       </c>
-      <c r="F30" s="116"/>
-      <c r="G30" s="116"/>
-      <c r="H30" s="116"/>
+      <c r="F30" s="118"/>
+      <c r="G30" s="118"/>
+      <c r="H30" s="118"/>
       <c r="L30" s="57"/>
       <c r="M30" s="57"/>
       <c r="N30" s="60"/>
@@ -2293,40 +2304,40 @@
       </c>
       <c r="C31" s="94"/>
       <c r="D31" s="95"/>
-      <c r="E31" s="115" t="s">
+      <c r="E31" s="117" t="s">
         <v>21</v>
       </c>
-      <c r="F31" s="115"/>
-      <c r="G31" s="115"/>
-      <c r="H31" s="115"/>
+      <c r="F31" s="117"/>
+      <c r="G31" s="117"/>
+      <c r="H31" s="117"/>
     </row>
     <row r="32" spans="1:19">
-      <c r="A32" s="115" t="s">
+      <c r="A32" s="117" t="s">
         <v>22</v>
       </c>
-      <c r="B32" s="115"/>
-      <c r="C32" s="115"/>
-      <c r="D32" s="115"/>
-      <c r="E32" s="115" t="s">
+      <c r="B32" s="117"/>
+      <c r="C32" s="117"/>
+      <c r="D32" s="117"/>
+      <c r="E32" s="117" t="s">
         <v>23</v>
       </c>
-      <c r="F32" s="115"/>
-      <c r="G32" s="115"/>
-      <c r="H32" s="115"/>
+      <c r="F32" s="117"/>
+      <c r="G32" s="117"/>
+      <c r="H32" s="117"/>
     </row>
     <row r="33" spans="1:8">
-      <c r="A33" s="115" t="s">
+      <c r="A33" s="117" t="s">
         <v>24</v>
       </c>
-      <c r="B33" s="115"/>
-      <c r="C33" s="115"/>
-      <c r="D33" s="115"/>
-      <c r="E33" s="115" t="s">
+      <c r="B33" s="117"/>
+      <c r="C33" s="117"/>
+      <c r="D33" s="117"/>
+      <c r="E33" s="117" t="s">
         <v>25</v>
       </c>
-      <c r="F33" s="115"/>
-      <c r="G33" s="115"/>
-      <c r="H33" s="115"/>
+      <c r="F33" s="117"/>
+      <c r="G33" s="117"/>
+      <c r="H33" s="117"/>
     </row>
     <row r="34" spans="1:8">
       <c r="A34" s="55"/>
@@ -2337,7 +2348,7 @@
       <c r="A35" s="63"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="43">
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="C22:G22"/>
     <mergeCell ref="A19:B19"/>
@@ -2353,6 +2364,11 @@
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="B10:C10"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="B6:D6"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="A28:H28"/>
@@ -2413,15 +2429,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="1" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A1" s="131" t="s">
+      <c r="A1" s="137" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="131"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
-      <c r="E1" s="131"/>
-      <c r="F1" s="131"/>
-      <c r="G1" s="131"/>
+      <c r="B1" s="137"/>
+      <c r="C1" s="137"/>
+      <c r="D1" s="137"/>
+      <c r="E1" s="137"/>
+      <c r="F1" s="137"/>
+      <c r="G1" s="137"/>
       <c r="M1" s="45"/>
       <c r="N1" s="45"/>
     </row>
@@ -2459,14 +2475,14 @@
     </row>
     <row r="5" spans="1:15" s="2" customFormat="1" ht="33" customHeight="1">
       <c r="A5" s="17"/>
-      <c r="B5" s="132" t="s">
+      <c r="B5" s="138" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="132"/>
-      <c r="D5" s="132"/>
-      <c r="E5" s="132"/>
-      <c r="F5" s="132"/>
-      <c r="G5" s="132"/>
+      <c r="C5" s="138"/>
+      <c r="D5" s="138"/>
+      <c r="E5" s="138"/>
+      <c r="F5" s="138"/>
+      <c r="G5" s="138"/>
       <c r="H5" s="18"/>
       <c r="M5" s="46"/>
       <c r="N5" s="46"/>
@@ -2486,27 +2502,27 @@
       <c r="A7" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="133" t="s">
+      <c r="B7" s="139" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="133"/>
-      <c r="D7" s="133"/>
-      <c r="E7" s="133"/>
-      <c r="F7" s="133"/>
+      <c r="C7" s="139"/>
+      <c r="D7" s="139"/>
+      <c r="E7" s="139"/>
+      <c r="F7" s="139"/>
       <c r="G7" s="20"/>
       <c r="M7" s="46"/>
       <c r="N7" s="46"/>
     </row>
     <row r="8" spans="1:15" s="2" customFormat="1" ht="54" customHeight="1">
       <c r="A8" s="17"/>
-      <c r="B8" s="134" t="s">
+      <c r="B8" s="140" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="134"/>
-      <c r="D8" s="134"/>
-      <c r="E8" s="134"/>
-      <c r="F8" s="134"/>
-      <c r="G8" s="134"/>
+      <c r="C8" s="140"/>
+      <c r="D8" s="140"/>
+      <c r="E8" s="140"/>
+      <c r="F8" s="140"/>
+      <c r="G8" s="140"/>
       <c r="M8" s="46"/>
       <c r="N8" s="46"/>
     </row>
@@ -2522,28 +2538,28 @@
       <c r="N9" s="46"/>
     </row>
     <row r="10" spans="1:15" s="3" customFormat="1" ht="49.5" customHeight="1">
-      <c r="A10" s="135" t="s">
+      <c r="A10" s="141" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="135"/>
-      <c r="C10" s="135"/>
-      <c r="D10" s="135"/>
-      <c r="E10" s="135"/>
-      <c r="F10" s="135"/>
-      <c r="G10" s="135"/>
+      <c r="B10" s="141"/>
+      <c r="C10" s="141"/>
+      <c r="D10" s="141"/>
+      <c r="E10" s="141"/>
+      <c r="F10" s="141"/>
+      <c r="G10" s="141"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
     </row>
     <row r="11" spans="1:15" s="3" customFormat="1" ht="27" customHeight="1">
-      <c r="A11" s="136" t="s">
+      <c r="A11" s="142" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="136"/>
-      <c r="C11" s="136"/>
-      <c r="D11" s="136"/>
-      <c r="E11" s="136"/>
-      <c r="F11" s="136"/>
-      <c r="G11" s="136"/>
+      <c r="B11" s="142"/>
+      <c r="C11" s="142"/>
+      <c r="D11" s="142"/>
+      <c r="E11" s="142"/>
+      <c r="F11" s="142"/>
+      <c r="G11" s="142"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
     </row>
@@ -2551,10 +2567,10 @@
       <c r="A12" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="137" t="s">
+      <c r="B12" s="143" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="138"/>
+      <c r="C12" s="144"/>
       <c r="D12" s="23" t="s">
         <v>5</v>
       </c>
@@ -2570,16 +2586,16 @@
       <c r="L12" s="47"/>
       <c r="M12" s="48"/>
       <c r="N12" s="49"/>
-      <c r="O12" s="149"/>
+      <c r="O12" s="155"/>
     </row>
     <row r="13" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1">
       <c r="A13" s="25">
         <v>1</v>
       </c>
-      <c r="B13" s="139">
+      <c r="B13" s="145">
         <v>50655</v>
       </c>
-      <c r="C13" s="140"/>
+      <c r="C13" s="146"/>
       <c r="D13" s="26" t="s">
         <v>7</v>
       </c>
@@ -2596,16 +2612,16 @@
       <c r="J13" s="51"/>
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
-      <c r="O13" s="149"/>
+      <c r="O13" s="155"/>
     </row>
     <row r="14" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1">
       <c r="A14" s="25">
         <v>2</v>
       </c>
-      <c r="B14" s="139">
+      <c r="B14" s="145">
         <v>50755</v>
       </c>
-      <c r="C14" s="140"/>
+      <c r="C14" s="146"/>
       <c r="D14" s="26" t="s">
         <v>8</v>
       </c>
@@ -2628,10 +2644,10 @@
       <c r="A15" s="25">
         <v>3</v>
       </c>
-      <c r="B15" s="139">
+      <c r="B15" s="145">
         <v>50665</v>
       </c>
-      <c r="C15" s="140"/>
+      <c r="C15" s="146"/>
       <c r="D15" s="26" t="s">
         <v>9</v>
       </c>
@@ -2654,10 +2670,10 @@
       <c r="A16" s="25">
         <v>4</v>
       </c>
-      <c r="B16" s="139">
+      <c r="B16" s="145">
         <v>50765</v>
       </c>
-      <c r="C16" s="140"/>
+      <c r="C16" s="146"/>
       <c r="D16" s="26" t="s">
         <v>10</v>
       </c>
@@ -2680,10 +2696,10 @@
       <c r="A17" s="25">
         <v>5</v>
       </c>
-      <c r="B17" s="139">
+      <c r="B17" s="145">
         <v>50720</v>
       </c>
-      <c r="C17" s="140"/>
+      <c r="C17" s="146"/>
       <c r="D17" s="26" t="s">
         <v>11</v>
       </c>
@@ -2706,10 +2722,10 @@
       <c r="A18" s="30">
         <v>6</v>
       </c>
-      <c r="B18" s="139">
+      <c r="B18" s="145">
         <v>50730</v>
       </c>
-      <c r="C18" s="140"/>
+      <c r="C18" s="146"/>
       <c r="D18" s="31" t="s">
         <v>12</v>
       </c>
@@ -2729,54 +2745,54 @@
       <c r="O18" s="50"/>
     </row>
     <row r="19" spans="1:15" s="4" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A19" s="150" t="s">
+      <c r="A19" s="156" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="151"/>
-      <c r="C19" s="152"/>
+      <c r="B19" s="157"/>
+      <c r="C19" s="158"/>
       <c r="D19" s="32"/>
-      <c r="E19" s="143">
+      <c r="E19" s="149">
         <f>SUM(E13:E18)</f>
         <v>6000</v>
       </c>
-      <c r="F19" s="145"/>
-      <c r="G19" s="147">
+      <c r="F19" s="151"/>
+      <c r="G19" s="153">
         <f>SUM(G13:G18)</f>
         <v>73120</v>
       </c>
       <c r="H19" s="33"/>
     </row>
     <row r="20" spans="1:15" s="4" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A20" s="153"/>
-      <c r="B20" s="154"/>
-      <c r="C20" s="155"/>
+      <c r="A20" s="159"/>
+      <c r="B20" s="160"/>
+      <c r="C20" s="161"/>
       <c r="D20" s="34"/>
-      <c r="E20" s="144"/>
-      <c r="F20" s="146"/>
-      <c r="G20" s="148"/>
+      <c r="E20" s="150"/>
+      <c r="F20" s="152"/>
+      <c r="G20" s="154"/>
     </row>
     <row r="21" spans="1:15" s="4" customFormat="1" ht="30" hidden="1" customHeight="1">
-      <c r="A21" s="141" t="s">
+      <c r="A21" s="147" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="141"/>
-      <c r="C21" s="141"/>
-      <c r="D21" s="141"/>
-      <c r="E21" s="141"/>
-      <c r="F21" s="141"/>
-      <c r="G21" s="141"/>
+      <c r="B21" s="147"/>
+      <c r="C21" s="147"/>
+      <c r="D21" s="147"/>
+      <c r="E21" s="147"/>
+      <c r="F21" s="147"/>
+      <c r="G21" s="147"/>
       <c r="J21" s="52"/>
     </row>
     <row r="22" spans="1:15" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A22" s="142" t="s">
+      <c r="A22" s="148" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="142"/>
-      <c r="C22" s="142"/>
-      <c r="D22" s="142"/>
-      <c r="E22" s="142"/>
-      <c r="F22" s="142"/>
-      <c r="G22" s="142"/>
+      <c r="B22" s="148"/>
+      <c r="C22" s="148"/>
+      <c r="D22" s="148"/>
+      <c r="E22" s="148"/>
+      <c r="F22" s="148"/>
+      <c r="G22" s="148"/>
       <c r="J22" s="52"/>
     </row>
     <row r="23" spans="1:15" s="4" customFormat="1" ht="21.75" customHeight="1">
@@ -2826,15 +2842,15 @@
       <c r="J26" s="52"/>
     </row>
     <row r="27" spans="1:15" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A27" s="142" t="s">
+      <c r="A27" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="142"/>
-      <c r="C27" s="142"/>
-      <c r="D27" s="142"/>
-      <c r="E27" s="142"/>
-      <c r="F27" s="142"/>
-      <c r="G27" s="142"/>
+      <c r="B27" s="148"/>
+      <c r="C27" s="148"/>
+      <c r="D27" s="148"/>
+      <c r="E27" s="148"/>
+      <c r="F27" s="148"/>
+      <c r="G27" s="148"/>
       <c r="J27" s="52"/>
     </row>
     <row r="28" spans="1:15" s="5" customFormat="1" ht="19.5" customHeight="1">
@@ -2898,15 +2914,15 @@
       <c r="N33" s="54"/>
     </row>
     <row r="34" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A34" s="142" t="s">
+      <c r="A34" s="148" t="s">
         <v>49</v>
       </c>
-      <c r="B34" s="142"/>
-      <c r="C34" s="142"/>
-      <c r="D34" s="142"/>
-      <c r="E34" s="142"/>
-      <c r="F34" s="142"/>
-      <c r="G34" s="142"/>
+      <c r="B34" s="148"/>
+      <c r="C34" s="148"/>
+      <c r="D34" s="148"/>
+      <c r="E34" s="148"/>
+      <c r="F34" s="148"/>
+      <c r="G34" s="148"/>
       <c r="J34" s="52"/>
     </row>
     <row r="35" spans="1:14" s="5" customFormat="1" ht="19.5" customHeight="1">
@@ -2930,15 +2946,15 @@
       <c r="N36" s="53"/>
     </row>
     <row r="37" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A37" s="142" t="s">
+      <c r="A37" s="148" t="s">
         <v>52</v>
       </c>
-      <c r="B37" s="142"/>
-      <c r="C37" s="142"/>
-      <c r="D37" s="142"/>
-      <c r="E37" s="142"/>
-      <c r="F37" s="142"/>
-      <c r="G37" s="142"/>
+      <c r="B37" s="148"/>
+      <c r="C37" s="148"/>
+      <c r="D37" s="148"/>
+      <c r="E37" s="148"/>
+      <c r="F37" s="148"/>
+      <c r="G37" s="148"/>
       <c r="J37" s="52"/>
     </row>
     <row r="38" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
@@ -2962,40 +2978,40 @@
       <c r="N39" s="54"/>
     </row>
     <row r="40" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A40" s="142" t="s">
+      <c r="A40" s="148" t="s">
         <v>55</v>
       </c>
-      <c r="B40" s="142"/>
-      <c r="C40" s="142"/>
-      <c r="D40" s="142"/>
-      <c r="E40" s="142"/>
-      <c r="F40" s="142"/>
-      <c r="G40" s="142"/>
+      <c r="B40" s="148"/>
+      <c r="C40" s="148"/>
+      <c r="D40" s="148"/>
+      <c r="E40" s="148"/>
+      <c r="F40" s="148"/>
+      <c r="G40" s="148"/>
       <c r="J40" s="52"/>
     </row>
     <row r="41" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A41" s="160" t="s">
+      <c r="A41" s="166" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="160"/>
-      <c r="C41" s="160"/>
-      <c r="D41" s="160"/>
-      <c r="E41" s="160"/>
-      <c r="F41" s="160"/>
-      <c r="G41" s="160"/>
+      <c r="B41" s="166"/>
+      <c r="C41" s="166"/>
+      <c r="D41" s="166"/>
+      <c r="E41" s="166"/>
+      <c r="F41" s="166"/>
+      <c r="G41" s="166"/>
       <c r="M41" s="54"/>
       <c r="N41" s="54"/>
     </row>
     <row r="42" spans="1:14" s="6" customFormat="1" ht="44.25" customHeight="1">
-      <c r="A42" s="156" t="s">
+      <c r="A42" s="162" t="s">
         <v>57</v>
       </c>
-      <c r="B42" s="156"/>
-      <c r="C42" s="156"/>
-      <c r="D42" s="156"/>
-      <c r="E42" s="156"/>
-      <c r="F42" s="156"/>
-      <c r="G42" s="156"/>
+      <c r="B42" s="162"/>
+      <c r="C42" s="162"/>
+      <c r="D42" s="162"/>
+      <c r="E42" s="162"/>
+      <c r="F42" s="162"/>
+      <c r="G42" s="162"/>
       <c r="M42" s="54"/>
       <c r="N42" s="54"/>
     </row>
@@ -3010,27 +3026,27 @@
       <c r="J43" s="52"/>
     </row>
     <row r="44" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A44" s="142" t="s">
+      <c r="A44" s="148" t="s">
         <v>58</v>
       </c>
-      <c r="B44" s="142"/>
-      <c r="C44" s="142"/>
-      <c r="D44" s="142"/>
-      <c r="E44" s="142"/>
-      <c r="F44" s="142"/>
-      <c r="G44" s="142"/>
+      <c r="B44" s="148"/>
+      <c r="C44" s="148"/>
+      <c r="D44" s="148"/>
+      <c r="E44" s="148"/>
+      <c r="F44" s="148"/>
+      <c r="G44" s="148"/>
       <c r="J44" s="52"/>
     </row>
     <row r="45" spans="1:14" s="6" customFormat="1" ht="58.5" customHeight="1">
-      <c r="A45" s="157" t="s">
+      <c r="A45" s="163" t="s">
         <v>59</v>
       </c>
-      <c r="B45" s="158"/>
-      <c r="C45" s="158"/>
-      <c r="D45" s="158"/>
-      <c r="E45" s="158"/>
-      <c r="F45" s="158"/>
-      <c r="G45" s="158"/>
+      <c r="B45" s="164"/>
+      <c r="C45" s="164"/>
+      <c r="D45" s="164"/>
+      <c r="E45" s="164"/>
+      <c r="F45" s="164"/>
+      <c r="G45" s="164"/>
       <c r="M45" s="54"/>
       <c r="N45" s="54"/>
     </row>
@@ -3045,27 +3061,27 @@
       <c r="J46" s="52"/>
     </row>
     <row r="47" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A47" s="142" t="s">
+      <c r="A47" s="148" t="s">
         <v>60</v>
       </c>
-      <c r="B47" s="142"/>
-      <c r="C47" s="142"/>
-      <c r="D47" s="142"/>
-      <c r="E47" s="142"/>
-      <c r="F47" s="142"/>
-      <c r="G47" s="142"/>
+      <c r="B47" s="148"/>
+      <c r="C47" s="148"/>
+      <c r="D47" s="148"/>
+      <c r="E47" s="148"/>
+      <c r="F47" s="148"/>
+      <c r="G47" s="148"/>
       <c r="J47" s="52"/>
     </row>
     <row r="48" spans="1:14" s="6" customFormat="1" ht="46.5" customHeight="1">
-      <c r="A48" s="159" t="s">
+      <c r="A48" s="165" t="s">
         <v>61</v>
       </c>
-      <c r="B48" s="159"/>
-      <c r="C48" s="159"/>
-      <c r="D48" s="159"/>
-      <c r="E48" s="159"/>
-      <c r="F48" s="159"/>
-      <c r="G48" s="159"/>
+      <c r="B48" s="165"/>
+      <c r="C48" s="165"/>
+      <c r="D48" s="165"/>
+      <c r="E48" s="165"/>
+      <c r="F48" s="165"/>
+      <c r="G48" s="165"/>
       <c r="M48" s="54"/>
       <c r="N48" s="54"/>
     </row>
@@ -3078,15 +3094,15 @@
       <c r="N49" s="54"/>
     </row>
     <row r="50" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A50" s="142" t="s">
+      <c r="A50" s="148" t="s">
         <v>62</v>
       </c>
-      <c r="B50" s="142"/>
-      <c r="C50" s="142"/>
-      <c r="D50" s="142"/>
-      <c r="E50" s="142"/>
-      <c r="F50" s="142"/>
-      <c r="G50" s="142"/>
+      <c r="B50" s="148"/>
+      <c r="C50" s="148"/>
+      <c r="D50" s="148"/>
+      <c r="E50" s="148"/>
+      <c r="F50" s="148"/>
+      <c r="G50" s="148"/>
       <c r="M50" s="54"/>
       <c r="N50" s="54"/>
     </row>

</xml_diff>

<commit_message>
feat: implement order and product management modules including detail, edit, and creation workflows with Excel PI export support.
</commit_message>
<xml_diff>
--- a/excel-template/PI-template.xlsx
+++ b/excel-template/PI-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\exportcrm\excel-template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2818FCBC-5192-4563-8666-69B64136EFF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B6C217-F013-4A72-81AC-51BCEB7D3345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -357,10 +357,6 @@
     <phoneticPr fontId="15" type="noConversion"/>
   </si>
   <si>
-    <t>0897</t>
-    <phoneticPr fontId="15" type="noConversion"/>
-  </si>
-  <si>
     <t>26-00336</t>
     <phoneticPr fontId="15" type="noConversion"/>
   </si>
@@ -467,6 +463,10 @@
   </si>
   <si>
     <t>0080-2062-0843</t>
+    <phoneticPr fontId="15" type="noConversion"/>
+  </si>
+  <si>
+    <t>0897</t>
     <phoneticPr fontId="15" type="noConversion"/>
   </si>
 </sst>
@@ -488,7 +488,7 @@
     <numFmt numFmtId="185" formatCode="_ * #,##0.00000_ ;_ * \-#,##0.00000_ ;_ * &quot;-&quot;??.000_ ;_ @_ "/>
     <numFmt numFmtId="186" formatCode="[$EUR]\ #,##0.00;[Red][$EUR]\ #,##0.00"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -909,7 +909,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="168">
+  <cellXfs count="167">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1168,9 +1168,6 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="185" fontId="20" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1253,6 +1250,9 @@
     <xf numFmtId="180" fontId="20" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -1272,7 +1272,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="186" fontId="21" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -1283,9 +1283,6 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="43" fontId="21" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1307,11 +1304,8 @@
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="20" fillId="0" borderId="16" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="43" fontId="17" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1403,8 +1397,11 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="17" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1754,9 +1751,9 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.33203125" style="96" customWidth="1"/>
+    <col min="1" max="1" width="6.33203125" style="95" customWidth="1"/>
     <col min="2" max="2" width="16.33203125" style="57" customWidth="1"/>
     <col min="3" max="3" width="8.44140625" style="57" customWidth="1"/>
     <col min="4" max="4" width="25.77734375" style="57" customWidth="1"/>
@@ -1777,69 +1774,69 @@
     <col min="19" max="16384" width="9" style="57"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="55" customFormat="1" ht="66" customHeight="1">
-      <c r="A1" s="102"/>
-      <c r="B1" s="102"/>
-      <c r="C1" s="102"/>
-      <c r="D1" s="102"/>
-      <c r="E1" s="102"/>
-      <c r="F1" s="130" t="s">
+    <row r="1" spans="1:19" s="55" customFormat="1" ht="66" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="101"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="129" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="130"/>
-      <c r="H1" s="130"/>
+      <c r="G1" s="129"/>
+      <c r="H1" s="129"/>
       <c r="N1" s="56"/>
       <c r="O1" s="56"/>
     </row>
-    <row r="2" spans="1:19" ht="21.9" customHeight="1">
-      <c r="A2" s="103" t="s">
+    <row r="2" spans="1:19" ht="21.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="102" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="95"/>
-      <c r="D2" s="95"/>
-      <c r="E2" s="95"/>
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
       <c r="F2" s="82" t="s">
         <v>80</v>
       </c>
-      <c r="G2" s="134" t="s">
-        <v>86</v>
-      </c>
-      <c r="H2" s="134"/>
-    </row>
-    <row r="3" spans="1:19" s="61" customFormat="1" ht="21.9" customHeight="1">
-      <c r="A3" s="104" t="s">
+      <c r="G2" s="133" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="133"/>
+    </row>
+    <row r="3" spans="1:19" s="61" customFormat="1" ht="21.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="103" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="105"/>
+      <c r="B3" s="104"/>
       <c r="C3" s="78"/>
       <c r="D3" s="77"/>
       <c r="E3" s="77"/>
       <c r="F3" s="82" t="s">
         <v>69</v>
       </c>
-      <c r="G3" s="135" t="s">
-        <v>87</v>
-      </c>
-      <c r="H3" s="135"/>
+      <c r="G3" s="165" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="165"/>
       <c r="N3" s="62"/>
       <c r="O3" s="62"/>
     </row>
-    <row r="4" spans="1:19" s="61" customFormat="1" ht="21.9" customHeight="1">
-      <c r="A4" s="101" t="s">
+    <row r="4" spans="1:19" s="61" customFormat="1" ht="21.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="100" t="s">
         <v>73</v>
       </c>
-      <c r="B4" s="105"/>
+      <c r="B4" s="104"/>
       <c r="C4" s="78"/>
       <c r="D4" s="77"/>
       <c r="E4" s="77"/>
       <c r="F4" s="82" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="135" t="s">
-        <v>88</v>
-      </c>
-      <c r="H4" s="135"/>
+      <c r="G4" s="165" t="s">
+        <v>87</v>
+      </c>
+      <c r="H4" s="165"/>
       <c r="J4" s="64"/>
       <c r="K4" s="65"/>
       <c r="L4" s="64"/>
@@ -1849,19 +1846,19 @@
       <c r="P4" s="67"/>
       <c r="Q4" s="67"/>
     </row>
-    <row r="5" spans="1:19" s="61" customFormat="1" ht="21.75" customHeight="1" thickBot="1">
-      <c r="A5" s="106"/>
-      <c r="B5" s="107"/>
-      <c r="C5" s="108"/>
-      <c r="D5" s="109"/>
-      <c r="E5" s="109"/>
-      <c r="F5" s="110" t="s">
+    <row r="5" spans="1:19" s="61" customFormat="1" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="105"/>
+      <c r="B5" s="106"/>
+      <c r="C5" s="107"/>
+      <c r="D5" s="108"/>
+      <c r="E5" s="108"/>
+      <c r="F5" s="109" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="136" t="s">
-        <v>89</v>
-      </c>
-      <c r="H5" s="136"/>
+      <c r="G5" s="166" t="s">
+        <v>88</v>
+      </c>
+      <c r="H5" s="166"/>
       <c r="J5" s="64"/>
       <c r="K5" s="65"/>
       <c r="L5" s="64"/>
@@ -1871,19 +1868,19 @@
       <c r="P5" s="67"/>
       <c r="Q5" s="67"/>
     </row>
-    <row r="6" spans="1:19" s="66" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A6" s="97" t="s">
+    <row r="6" spans="1:19" s="66" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="96" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="167" t="s">
+      <c r="B6" s="134" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="167"/>
-      <c r="D6" s="167"/>
+      <c r="C6" s="134"/>
+      <c r="D6" s="134"/>
       <c r="E6" s="68"/>
-      <c r="F6" s="99"/>
-      <c r="G6" s="100"/>
-      <c r="H6" s="100"/>
+      <c r="F6" s="98"/>
+      <c r="G6" s="99"/>
+      <c r="H6" s="99"/>
       <c r="I6" s="69"/>
       <c r="J6" s="70"/>
       <c r="K6" s="70"/>
@@ -1895,19 +1892,19 @@
       <c r="Q6" s="70"/>
       <c r="R6" s="70"/>
     </row>
-    <row r="7" spans="1:19" s="66" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="7" spans="1:19" s="66" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="76" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="131" t="s">
+      <c r="B7" s="130" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="131"/>
-      <c r="D7" s="131"/>
-      <c r="E7" s="98"/>
-      <c r="F7" s="129"/>
-      <c r="G7" s="129"/>
-      <c r="H7" s="129"/>
+      <c r="C7" s="130"/>
+      <c r="D7" s="130"/>
+      <c r="E7" s="97"/>
+      <c r="F7" s="128"/>
+      <c r="G7" s="128"/>
+      <c r="H7" s="128"/>
       <c r="I7" s="67"/>
       <c r="J7" s="73"/>
       <c r="K7" s="67"/>
@@ -1919,19 +1916,19 @@
       <c r="Q7" s="75"/>
       <c r="R7" s="73"/>
     </row>
-    <row r="8" spans="1:19" s="66" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="8" spans="1:19" s="66" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="76" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="131" t="s">
+      <c r="B8" s="130" t="s">
         <v>79</v>
       </c>
-      <c r="C8" s="131"/>
-      <c r="D8" s="131"/>
-      <c r="E8" s="98"/>
-      <c r="F8" s="129"/>
-      <c r="G8" s="129"/>
-      <c r="H8" s="129"/>
+      <c r="C8" s="130"/>
+      <c r="D8" s="130"/>
+      <c r="E8" s="97"/>
+      <c r="F8" s="128"/>
+      <c r="G8" s="128"/>
+      <c r="H8" s="128"/>
       <c r="I8" s="64"/>
       <c r="J8" s="64"/>
       <c r="K8" s="64"/>
@@ -1943,82 +1940,82 @@
       <c r="Q8" s="75"/>
       <c r="R8" s="73"/>
     </row>
-    <row r="9" spans="1:19" s="78" customFormat="1" ht="23.25" customHeight="1">
-      <c r="A9" s="132" t="s">
+    <row r="9" spans="1:19" s="78" customFormat="1" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="131" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="132"/>
-      <c r="C9" s="132"/>
-      <c r="D9" s="132"/>
-      <c r="E9" s="132"/>
-      <c r="F9" s="132"/>
-      <c r="G9" s="132"/>
-      <c r="H9" s="132"/>
+      <c r="B9" s="131"/>
+      <c r="C9" s="131"/>
+      <c r="D9" s="131"/>
+      <c r="E9" s="131"/>
+      <c r="F9" s="131"/>
+      <c r="G9" s="131"/>
+      <c r="H9" s="131"/>
       <c r="I9" s="77"/>
       <c r="J9" s="77"/>
       <c r="K9" s="77"/>
-      <c r="L9" s="128"/>
-      <c r="M9" s="128"/>
-      <c r="N9" s="128"/>
-      <c r="O9" s="128"/>
-      <c r="P9" s="128"/>
-      <c r="Q9" s="128"/>
-      <c r="R9" s="128"/>
-      <c r="S9" s="128"/>
-    </row>
-    <row r="10" spans="1:19" s="79" customFormat="1" ht="26.25" customHeight="1">
-      <c r="A10" s="111" t="s">
+      <c r="L9" s="127"/>
+      <c r="M9" s="127"/>
+      <c r="N9" s="127"/>
+      <c r="O9" s="127"/>
+      <c r="P9" s="127"/>
+      <c r="Q9" s="127"/>
+      <c r="R9" s="127"/>
+      <c r="S9" s="127"/>
+    </row>
+    <row r="10" spans="1:19" s="79" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="110" t="s">
         <v>3</v>
       </c>
-      <c r="B10" s="133" t="s">
+      <c r="B10" s="132" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="133"/>
-      <c r="D10" s="111" t="s">
+      <c r="C10" s="132"/>
+      <c r="D10" s="110" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="111" t="s">
+      <c r="E10" s="110" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="111" t="s">
-        <v>90</v>
-      </c>
-      <c r="G10" s="111" t="s">
+      <c r="F10" s="110" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" s="110" t="s">
         <v>82</v>
       </c>
-      <c r="H10" s="111" t="s">
+      <c r="H10" s="110" t="s">
         <v>83</v>
       </c>
-      <c r="L10" s="128"/>
-      <c r="M10" s="128"/>
-      <c r="N10" s="128"/>
-      <c r="O10" s="128"/>
-      <c r="P10" s="128"/>
-      <c r="Q10" s="128"/>
-      <c r="R10" s="128"/>
-      <c r="S10" s="128"/>
-    </row>
-    <row r="11" spans="1:19" s="78" customFormat="1" ht="20.100000000000001" customHeight="1">
+      <c r="L10" s="127"/>
+      <c r="M10" s="127"/>
+      <c r="N10" s="127"/>
+      <c r="O10" s="127"/>
+      <c r="P10" s="127"/>
+      <c r="Q10" s="127"/>
+      <c r="R10" s="127"/>
+      <c r="S10" s="127"/>
+    </row>
+    <row r="11" spans="1:19" s="78" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="80">
         <v>1</v>
       </c>
       <c r="B11" s="119" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C11" s="119"/>
-      <c r="D11" s="113" t="s">
-        <v>112</v>
-      </c>
-      <c r="E11" s="114">
+      <c r="D11" s="112" t="s">
+        <v>111</v>
+      </c>
+      <c r="E11" s="113">
         <v>250</v>
       </c>
-      <c r="F11" s="114" t="s">
-        <v>91</v>
-      </c>
-      <c r="G11" s="115">
+      <c r="F11" s="113" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="114">
         <v>14.3</v>
       </c>
-      <c r="H11" s="116">
+      <c r="H11" s="115">
         <v>3575</v>
       </c>
       <c r="K11" s="81"/>
@@ -2027,7 +2024,7 @@
       <c r="P11" s="82"/>
       <c r="Q11" s="82"/>
     </row>
-    <row r="12" spans="1:19" s="77" customFormat="1" ht="16.5" customHeight="1">
+    <row r="12" spans="1:19" s="77" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="80" t="s">
         <v>68</v>
       </c>
@@ -2035,11 +2032,11 @@
       <c r="C12" s="80"/>
       <c r="D12" s="80"/>
       <c r="E12" s="80"/>
-      <c r="F12" s="112" t="s">
+      <c r="F12" s="111" t="s">
         <v>14</v>
       </c>
       <c r="G12" s="122" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H12" s="123">
         <f>SUM(H11:H11)</f>
@@ -2047,17 +2044,17 @@
       </c>
       <c r="I12" s="83"/>
     </row>
-    <row r="13" spans="1:19" s="77" customFormat="1" ht="13.5" customHeight="1">
+    <row r="13" spans="1:19" s="77" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="80"/>
       <c r="B13" s="80"/>
       <c r="C13" s="80"/>
       <c r="D13" s="80"/>
       <c r="E13" s="80"/>
-      <c r="F13" s="112"/>
+      <c r="F13" s="111"/>
       <c r="G13" s="122"/>
       <c r="H13" s="123"/>
     </row>
-    <row r="14" spans="1:19" s="77" customFormat="1" ht="30" customHeight="1">
+    <row r="14" spans="1:19" s="77" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="126" t="s">
         <v>84</v>
       </c>
@@ -2070,13 +2067,13 @@
       <c r="H14" s="126"/>
       <c r="K14" s="84"/>
     </row>
-    <row r="15" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="15" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="124" t="s">
         <v>85</v>
       </c>
       <c r="B15" s="124"/>
       <c r="C15" s="124" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D15" s="124"/>
       <c r="E15" s="124"/>
@@ -2085,13 +2082,13 @@
       <c r="H15" s="85"/>
       <c r="K15" s="84"/>
     </row>
-    <row r="16" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="16" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="124" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B16" s="124"/>
       <c r="C16" s="124" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D16" s="124"/>
       <c r="E16" s="124"/>
@@ -2100,13 +2097,13 @@
       <c r="H16" s="85"/>
       <c r="K16" s="84"/>
     </row>
-    <row r="17" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="17" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="124" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B17" s="124"/>
       <c r="C17" s="124" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D17" s="124"/>
       <c r="E17" s="124"/>
@@ -2115,72 +2112,72 @@
       <c r="H17" s="85"/>
       <c r="K17" s="84"/>
     </row>
-    <row r="18" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="18" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="124" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B18" s="124"/>
       <c r="C18" s="124" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D18" s="124"/>
       <c r="E18" s="124"/>
       <c r="F18" s="124"/>
       <c r="G18" s="124"/>
     </row>
-    <row r="19" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="19" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="124" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B19" s="124"/>
       <c r="C19" s="124" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D19" s="124"/>
       <c r="E19" s="124"/>
       <c r="F19" s="124"/>
       <c r="G19" s="124"/>
     </row>
-    <row r="20" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="20" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="124" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B20" s="124"/>
       <c r="C20" s="124" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D20" s="124"/>
       <c r="E20" s="124"/>
       <c r="F20" s="124"/>
       <c r="G20" s="124"/>
     </row>
-    <row r="21" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="21" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="124" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B21" s="124"/>
       <c r="C21" s="124" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D21" s="124"/>
       <c r="E21" s="124"/>
       <c r="F21" s="124"/>
       <c r="G21" s="124"/>
     </row>
-    <row r="22" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="22" spans="1:19" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="124" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B22" s="124"/>
       <c r="C22" s="124" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D22" s="124"/>
       <c r="E22" s="124"/>
       <c r="F22" s="124"/>
       <c r="G22" s="124"/>
     </row>
-    <row r="23" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1">
+    <row r="23" spans="1:19" s="77" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="72"/>
       <c r="B23" s="72"/>
       <c r="C23" s="72"/>
@@ -2191,9 +2188,9 @@
       <c r="H23" s="86"/>
       <c r="K23" s="84"/>
     </row>
-    <row r="24" spans="1:19" s="77" customFormat="1" ht="31.5" customHeight="1">
+    <row r="24" spans="1:19" s="77" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="125" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B24" s="125"/>
       <c r="C24" s="125"/>
@@ -2204,20 +2201,20 @@
       <c r="H24" s="125"/>
       <c r="K24" s="84"/>
     </row>
-    <row r="25" spans="1:19" s="70" customFormat="1" ht="20.100000000000001" customHeight="1">
-      <c r="A25" s="127" t="s">
-        <v>110</v>
-      </c>
-      <c r="B25" s="127"/>
-      <c r="C25" s="127"/>
-      <c r="D25" s="127"/>
-      <c r="E25" s="127"/>
-      <c r="F25" s="87"/>
-      <c r="G25" s="87"/>
-      <c r="H25" s="87"/>
-      <c r="K25" s="88"/>
-    </row>
-    <row r="26" spans="1:19" s="77" customFormat="1" ht="27" customHeight="1">
+    <row r="25" spans="1:19" s="70" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="116" t="s">
+        <v>109</v>
+      </c>
+      <c r="B25" s="116"/>
+      <c r="C25" s="116"/>
+      <c r="D25" s="116"/>
+      <c r="E25" s="116"/>
+      <c r="F25" s="116"/>
+      <c r="G25" s="116"/>
+      <c r="H25" s="116"/>
+      <c r="K25" s="87"/>
+    </row>
+    <row r="26" spans="1:19" s="77" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="72"/>
       <c r="B26" s="72"/>
       <c r="C26" s="72"/>
@@ -2227,18 +2224,18 @@
       <c r="G26" s="86"/>
       <c r="H26" s="86"/>
       <c r="K26" s="84"/>
-      <c r="L26" s="89"/>
-      <c r="M26" s="89"/>
-      <c r="N26" s="90"/>
-      <c r="O26" s="90"/>
-      <c r="P26" s="89"/>
-      <c r="Q26" s="89"/>
-      <c r="R26" s="89"/>
-      <c r="S26" s="89"/>
-    </row>
-    <row r="27" spans="1:19" s="89" customFormat="1" ht="19.5" customHeight="1">
+      <c r="L26" s="88"/>
+      <c r="M26" s="88"/>
+      <c r="N26" s="89"/>
+      <c r="O26" s="89"/>
+      <c r="P26" s="88"/>
+      <c r="Q26" s="88"/>
+      <c r="R26" s="88"/>
+      <c r="S26" s="88"/>
+    </row>
+    <row r="27" spans="1:19" s="88" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="120" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B27" s="120"/>
       <c r="C27" s="120"/>
@@ -2247,12 +2244,12 @@
       <c r="F27" s="120"/>
       <c r="G27" s="120"/>
       <c r="H27" s="120"/>
-      <c r="N27" s="90"/>
-      <c r="O27" s="90"/>
-    </row>
-    <row r="28" spans="1:19" s="89" customFormat="1" ht="53.25" customHeight="1">
+      <c r="N27" s="89"/>
+      <c r="O27" s="89"/>
+    </row>
+    <row r="28" spans="1:19" s="88" customFormat="1" ht="53.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="121" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B28" s="121"/>
       <c r="C28" s="121"/>
@@ -2261,22 +2258,22 @@
       <c r="F28" s="121"/>
       <c r="G28" s="121"/>
       <c r="H28" s="121"/>
-      <c r="N28" s="90"/>
-      <c r="O28" s="90"/>
-    </row>
-    <row r="29" spans="1:19" s="89" customFormat="1" ht="24" customHeight="1" thickBot="1">
-      <c r="A29" s="91"/>
-      <c r="B29" s="91"/>
-      <c r="C29" s="91"/>
-      <c r="D29" s="91"/>
-      <c r="E29" s="91"/>
-      <c r="F29" s="91"/>
-      <c r="G29" s="91"/>
-      <c r="H29" s="91"/>
-      <c r="N29" s="90"/>
-      <c r="O29" s="90"/>
-    </row>
-    <row r="30" spans="1:19" s="89" customFormat="1" ht="19.5" customHeight="1">
+      <c r="N28" s="89"/>
+      <c r="O28" s="89"/>
+    </row>
+    <row r="29" spans="1:19" s="88" customFormat="1" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="90"/>
+      <c r="B29" s="90"/>
+      <c r="C29" s="90"/>
+      <c r="D29" s="90"/>
+      <c r="E29" s="90"/>
+      <c r="F29" s="90"/>
+      <c r="G29" s="90"/>
+      <c r="H29" s="90"/>
+      <c r="N29" s="89"/>
+      <c r="O29" s="89"/>
+    </row>
+    <row r="30" spans="1:19" s="88" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="118" t="s">
         <v>18</v>
       </c>
@@ -2298,12 +2295,12 @@
       <c r="R30" s="57"/>
       <c r="S30" s="57"/>
     </row>
-    <row r="31" spans="1:19">
-      <c r="A31" s="93" t="s">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A31" s="92" t="s">
         <v>20</v>
       </c>
-      <c r="C31" s="94"/>
-      <c r="D31" s="95"/>
+      <c r="C31" s="93"/>
+      <c r="D31" s="94"/>
       <c r="E31" s="117" t="s">
         <v>21</v>
       </c>
@@ -2311,7 +2308,7 @@
       <c r="G31" s="117"/>
       <c r="H31" s="117"/>
     </row>
-    <row r="32" spans="1:19">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="117" t="s">
         <v>22</v>
       </c>
@@ -2325,7 +2322,7 @@
       <c r="G32" s="117"/>
       <c r="H32" s="117"/>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="117" t="s">
         <v>24</v>
       </c>
@@ -2339,17 +2336,16 @@
       <c r="G33" s="117"/>
       <c r="H33" s="117"/>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" s="55"/>
       <c r="F34" s="55"/>
-      <c r="H34" s="92"/>
-    </row>
-    <row r="35" spans="1:8">
+      <c r="H34" s="91"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="63"/>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="A22:B22"/>
     <mergeCell ref="C22:G22"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="C19:G19"/>
@@ -2384,7 +2380,8 @@
     <mergeCell ref="C16:G16"/>
     <mergeCell ref="C17:G17"/>
     <mergeCell ref="C18:G18"/>
-    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="E33:H33"/>
     <mergeCell ref="A32:D32"/>
     <mergeCell ref="A33:D33"/>
@@ -2408,7 +2405,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O54"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.21875" style="7" customWidth="1"/>
     <col min="2" max="2" width="7" style="8" customWidth="1"/>
@@ -2428,20 +2425,20 @@
     <col min="16" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="1" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A1" s="137" t="s">
+    <row r="1" spans="1:15" s="1" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="135" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="137"/>
-      <c r="C1" s="137"/>
-      <c r="D1" s="137"/>
-      <c r="E1" s="137"/>
-      <c r="F1" s="137"/>
-      <c r="G1" s="137"/>
+      <c r="B1" s="135"/>
+      <c r="C1" s="135"/>
+      <c r="D1" s="135"/>
+      <c r="E1" s="135"/>
+      <c r="F1" s="135"/>
+      <c r="G1" s="135"/>
       <c r="M1" s="45"/>
       <c r="N1" s="45"/>
     </row>
-    <row r="2" spans="1:15" ht="13.5" customHeight="1">
+    <row r="2" spans="1:15" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F2" s="12" t="s">
         <v>27</v>
       </c>
@@ -2452,7 +2449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15" customHeight="1">
+    <row r="3" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F3" s="12" t="s">
         <v>28</v>
       </c>
@@ -2460,7 +2457,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>30</v>
       </c>
@@ -2473,21 +2470,21 @@
       <c r="G4" s="16"/>
       <c r="H4" s="9"/>
     </row>
-    <row r="5" spans="1:15" s="2" customFormat="1" ht="33" customHeight="1">
+    <row r="5" spans="1:15" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="17"/>
-      <c r="B5" s="138" t="s">
+      <c r="B5" s="136" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="138"/>
-      <c r="D5" s="138"/>
-      <c r="E5" s="138"/>
-      <c r="F5" s="138"/>
-      <c r="G5" s="138"/>
+      <c r="C5" s="136"/>
+      <c r="D5" s="136"/>
+      <c r="E5" s="136"/>
+      <c r="F5" s="136"/>
+      <c r="G5" s="136"/>
       <c r="H5" s="18"/>
       <c r="M5" s="46"/>
       <c r="N5" s="46"/>
     </row>
-    <row r="6" spans="1:15" s="2" customFormat="1" ht="5.25" customHeight="1">
+    <row r="6" spans="1:15" s="2" customFormat="1" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="17"/>
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
@@ -2498,35 +2495,35 @@
       <c r="M6" s="46"/>
       <c r="N6" s="46"/>
     </row>
-    <row r="7" spans="1:15" s="2" customFormat="1">
+    <row r="7" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="139" t="s">
+      <c r="B7" s="137" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="139"/>
-      <c r="D7" s="139"/>
-      <c r="E7" s="139"/>
-      <c r="F7" s="139"/>
+      <c r="C7" s="137"/>
+      <c r="D7" s="137"/>
+      <c r="E7" s="137"/>
+      <c r="F7" s="137"/>
       <c r="G7" s="20"/>
       <c r="M7" s="46"/>
       <c r="N7" s="46"/>
     </row>
-    <row r="8" spans="1:15" s="2" customFormat="1" ht="54" customHeight="1">
+    <row r="8" spans="1:15" s="2" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
-      <c r="B8" s="140" t="s">
+      <c r="B8" s="138" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="140"/>
-      <c r="D8" s="140"/>
-      <c r="E8" s="140"/>
-      <c r="F8" s="140"/>
-      <c r="G8" s="140"/>
+      <c r="C8" s="138"/>
+      <c r="D8" s="138"/>
+      <c r="E8" s="138"/>
+      <c r="F8" s="138"/>
+      <c r="G8" s="138"/>
       <c r="M8" s="46"/>
       <c r="N8" s="46"/>
     </row>
-    <row r="9" spans="1:15" s="2" customFormat="1" ht="6" customHeight="1">
+    <row r="9" spans="1:15" s="2" customFormat="1" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="17"/>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -2537,40 +2534,40 @@
       <c r="M9" s="46"/>
       <c r="N9" s="46"/>
     </row>
-    <row r="10" spans="1:15" s="3" customFormat="1" ht="49.5" customHeight="1">
-      <c r="A10" s="141" t="s">
+    <row r="10" spans="1:15" s="3" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="139" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="141"/>
-      <c r="C10" s="141"/>
-      <c r="D10" s="141"/>
-      <c r="E10" s="141"/>
-      <c r="F10" s="141"/>
-      <c r="G10" s="141"/>
+      <c r="B10" s="139"/>
+      <c r="C10" s="139"/>
+      <c r="D10" s="139"/>
+      <c r="E10" s="139"/>
+      <c r="F10" s="139"/>
+      <c r="G10" s="139"/>
       <c r="M10" s="4"/>
       <c r="N10" s="4"/>
     </row>
-    <row r="11" spans="1:15" s="3" customFormat="1" ht="27" customHeight="1">
-      <c r="A11" s="142" t="s">
+    <row r="11" spans="1:15" s="3" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="140" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="142"/>
-      <c r="C11" s="142"/>
-      <c r="D11" s="142"/>
-      <c r="E11" s="142"/>
-      <c r="F11" s="142"/>
-      <c r="G11" s="142"/>
+      <c r="B11" s="140"/>
+      <c r="C11" s="140"/>
+      <c r="D11" s="140"/>
+      <c r="E11" s="140"/>
+      <c r="F11" s="140"/>
+      <c r="G11" s="140"/>
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
     </row>
-    <row r="12" spans="1:15" s="4" customFormat="1" ht="30.75" customHeight="1">
+    <row r="12" spans="1:15" s="4" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="143" t="s">
+      <c r="B12" s="141" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="144"/>
+      <c r="C12" s="142"/>
       <c r="D12" s="23" t="s">
         <v>5</v>
       </c>
@@ -2586,16 +2583,16 @@
       <c r="L12" s="47"/>
       <c r="M12" s="48"/>
       <c r="N12" s="49"/>
-      <c r="O12" s="155"/>
-    </row>
-    <row r="13" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1">
+      <c r="O12" s="153"/>
+    </row>
+    <row r="13" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="25">
         <v>1</v>
       </c>
-      <c r="B13" s="145">
+      <c r="B13" s="143">
         <v>50655</v>
       </c>
-      <c r="C13" s="146"/>
+      <c r="C13" s="144"/>
       <c r="D13" s="26" t="s">
         <v>7</v>
       </c>
@@ -2612,16 +2609,16 @@
       <c r="J13" s="51"/>
       <c r="M13" s="4"/>
       <c r="N13" s="4"/>
-      <c r="O13" s="155"/>
-    </row>
-    <row r="14" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1">
+      <c r="O13" s="153"/>
+    </row>
+    <row r="14" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="25">
         <v>2</v>
       </c>
-      <c r="B14" s="145">
+      <c r="B14" s="143">
         <v>50755</v>
       </c>
-      <c r="C14" s="146"/>
+      <c r="C14" s="144"/>
       <c r="D14" s="26" t="s">
         <v>8</v>
       </c>
@@ -2640,14 +2637,14 @@
       <c r="N14" s="4"/>
       <c r="O14" s="50"/>
     </row>
-    <row r="15" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1">
+    <row r="15" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="25">
         <v>3</v>
       </c>
-      <c r="B15" s="145">
+      <c r="B15" s="143">
         <v>50665</v>
       </c>
-      <c r="C15" s="146"/>
+      <c r="C15" s="144"/>
       <c r="D15" s="26" t="s">
         <v>9</v>
       </c>
@@ -2666,14 +2663,14 @@
       <c r="N15" s="4"/>
       <c r="O15" s="50"/>
     </row>
-    <row r="16" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1">
+    <row r="16" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="25">
         <v>4</v>
       </c>
-      <c r="B16" s="145">
+      <c r="B16" s="143">
         <v>50765</v>
       </c>
-      <c r="C16" s="146"/>
+      <c r="C16" s="144"/>
       <c r="D16" s="26" t="s">
         <v>10</v>
       </c>
@@ -2692,14 +2689,14 @@
       <c r="N16" s="4"/>
       <c r="O16" s="50"/>
     </row>
-    <row r="17" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1">
+    <row r="17" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="25">
         <v>5</v>
       </c>
-      <c r="B17" s="145">
+      <c r="B17" s="143">
         <v>50720</v>
       </c>
-      <c r="C17" s="146"/>
+      <c r="C17" s="144"/>
       <c r="D17" s="26" t="s">
         <v>11</v>
       </c>
@@ -2718,14 +2715,14 @@
       <c r="N17" s="4"/>
       <c r="O17" s="50"/>
     </row>
-    <row r="18" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1">
+    <row r="18" spans="1:15" s="3" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="30">
         <v>6</v>
       </c>
-      <c r="B18" s="145">
+      <c r="B18" s="143">
         <v>50730</v>
       </c>
-      <c r="C18" s="146"/>
+      <c r="C18" s="144"/>
       <c r="D18" s="31" t="s">
         <v>12</v>
       </c>
@@ -2744,58 +2741,58 @@
       <c r="N18" s="4"/>
       <c r="O18" s="50"/>
     </row>
-    <row r="19" spans="1:15" s="4" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A19" s="156" t="s">
+    <row r="19" spans="1:15" s="4" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="154" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="157"/>
-      <c r="C19" s="158"/>
+      <c r="B19" s="155"/>
+      <c r="C19" s="156"/>
       <c r="D19" s="32"/>
-      <c r="E19" s="149">
+      <c r="E19" s="147">
         <f>SUM(E13:E18)</f>
         <v>6000</v>
       </c>
-      <c r="F19" s="151"/>
-      <c r="G19" s="153">
+      <c r="F19" s="149"/>
+      <c r="G19" s="151">
         <f>SUM(G13:G18)</f>
         <v>73120</v>
       </c>
       <c r="H19" s="33"/>
     </row>
-    <row r="20" spans="1:15" s="4" customFormat="1" ht="13.5" customHeight="1">
-      <c r="A20" s="159"/>
-      <c r="B20" s="160"/>
-      <c r="C20" s="161"/>
+    <row r="20" spans="1:15" s="4" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="157"/>
+      <c r="B20" s="158"/>
+      <c r="C20" s="159"/>
       <c r="D20" s="34"/>
-      <c r="E20" s="150"/>
-      <c r="F20" s="152"/>
-      <c r="G20" s="154"/>
-    </row>
-    <row r="21" spans="1:15" s="4" customFormat="1" ht="30" hidden="1" customHeight="1">
-      <c r="A21" s="147" t="s">
+      <c r="E20" s="148"/>
+      <c r="F20" s="150"/>
+      <c r="G20" s="152"/>
+    </row>
+    <row r="21" spans="1:15" s="4" customFormat="1" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="145" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="147"/>
-      <c r="C21" s="147"/>
-      <c r="D21" s="147"/>
-      <c r="E21" s="147"/>
-      <c r="F21" s="147"/>
-      <c r="G21" s="147"/>
+      <c r="B21" s="145"/>
+      <c r="C21" s="145"/>
+      <c r="D21" s="145"/>
+      <c r="E21" s="145"/>
+      <c r="F21" s="145"/>
+      <c r="G21" s="145"/>
       <c r="J21" s="52"/>
     </row>
-    <row r="22" spans="1:15" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A22" s="148" t="s">
+    <row r="22" spans="1:15" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="146" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="148"/>
-      <c r="C22" s="148"/>
-      <c r="D22" s="148"/>
-      <c r="E22" s="148"/>
-      <c r="F22" s="148"/>
-      <c r="G22" s="148"/>
+      <c r="B22" s="146"/>
+      <c r="C22" s="146"/>
+      <c r="D22" s="146"/>
+      <c r="E22" s="146"/>
+      <c r="F22" s="146"/>
+      <c r="G22" s="146"/>
       <c r="J22" s="52"/>
     </row>
-    <row r="23" spans="1:15" s="4" customFormat="1" ht="21.75" customHeight="1">
+    <row r="23" spans="1:15" s="4" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="36" t="s">
         <v>15</v>
       </c>
@@ -2807,7 +2804,7 @@
       <c r="G23" s="35"/>
       <c r="J23" s="52"/>
     </row>
-    <row r="24" spans="1:15" s="4" customFormat="1" ht="21.75" customHeight="1">
+    <row r="24" spans="1:15" s="4" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="36" t="s">
         <v>16</v>
       </c>
@@ -2819,7 +2816,7 @@
       <c r="G24" s="35"/>
       <c r="J24" s="52"/>
     </row>
-    <row r="25" spans="1:15" s="4" customFormat="1" ht="21.75" customHeight="1">
+    <row r="25" spans="1:15" s="4" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="36" t="s">
         <v>17</v>
       </c>
@@ -2831,7 +2828,7 @@
       <c r="G25" s="35"/>
       <c r="J25" s="52"/>
     </row>
-    <row r="26" spans="1:15" s="4" customFormat="1" ht="1.5" customHeight="1">
+    <row r="26" spans="1:15" s="4" customFormat="1" ht="1.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="35"/>
       <c r="B26" s="35"/>
       <c r="C26" s="35"/>
@@ -2841,19 +2838,19 @@
       <c r="G26" s="35"/>
       <c r="J26" s="52"/>
     </row>
-    <row r="27" spans="1:15" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A27" s="148" t="s">
+    <row r="27" spans="1:15" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="146" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="148"/>
-      <c r="C27" s="148"/>
-      <c r="D27" s="148"/>
-      <c r="E27" s="148"/>
-      <c r="F27" s="148"/>
-      <c r="G27" s="148"/>
+      <c r="B27" s="146"/>
+      <c r="C27" s="146"/>
+      <c r="D27" s="146"/>
+      <c r="E27" s="146"/>
+      <c r="F27" s="146"/>
+      <c r="G27" s="146"/>
       <c r="J27" s="52"/>
     </row>
-    <row r="28" spans="1:15" s="5" customFormat="1" ht="19.5" customHeight="1">
+    <row r="28" spans="1:15" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="36" t="s">
         <v>43</v>
       </c>
@@ -2863,7 +2860,7 @@
       <c r="M28" s="53"/>
       <c r="N28" s="53"/>
     </row>
-    <row r="29" spans="1:15" s="5" customFormat="1" ht="19.5" customHeight="1">
+    <row r="29" spans="1:15" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="36" t="s">
         <v>44</v>
       </c>
@@ -2873,7 +2870,7 @@
       <c r="M29" s="53"/>
       <c r="N29" s="53"/>
     </row>
-    <row r="30" spans="1:15" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="30" spans="1:15" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="36" t="s">
         <v>45</v>
       </c>
@@ -2883,7 +2880,7 @@
       <c r="M30" s="54"/>
       <c r="N30" s="54"/>
     </row>
-    <row r="31" spans="1:15" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="31" spans="1:15" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="36" t="s">
         <v>46</v>
       </c>
@@ -2893,7 +2890,7 @@
       <c r="M31" s="54"/>
       <c r="N31" s="54"/>
     </row>
-    <row r="32" spans="1:15" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="32" spans="1:15" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="36" t="s">
         <v>47</v>
       </c>
@@ -2903,7 +2900,7 @@
       <c r="M32" s="54"/>
       <c r="N32" s="54"/>
     </row>
-    <row r="33" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="33" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="36" t="s">
         <v>48</v>
       </c>
@@ -2913,19 +2910,19 @@
       <c r="M33" s="54"/>
       <c r="N33" s="54"/>
     </row>
-    <row r="34" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A34" s="148" t="s">
+    <row r="34" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="B34" s="148"/>
-      <c r="C34" s="148"/>
-      <c r="D34" s="148"/>
-      <c r="E34" s="148"/>
-      <c r="F34" s="148"/>
-      <c r="G34" s="148"/>
+      <c r="B34" s="146"/>
+      <c r="C34" s="146"/>
+      <c r="D34" s="146"/>
+      <c r="E34" s="146"/>
+      <c r="F34" s="146"/>
+      <c r="G34" s="146"/>
       <c r="J34" s="52"/>
     </row>
-    <row r="35" spans="1:14" s="5" customFormat="1" ht="19.5" customHeight="1">
+    <row r="35" spans="1:14" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="36" t="s">
         <v>50</v>
       </c>
@@ -2935,7 +2932,7 @@
       <c r="M35" s="53"/>
       <c r="N35" s="53"/>
     </row>
-    <row r="36" spans="1:14" s="5" customFormat="1" ht="19.5" customHeight="1">
+    <row r="36" spans="1:14" s="5" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="36" t="s">
         <v>51</v>
       </c>
@@ -2945,19 +2942,19 @@
       <c r="M36" s="53"/>
       <c r="N36" s="53"/>
     </row>
-    <row r="37" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A37" s="148" t="s">
+    <row r="37" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="146" t="s">
         <v>52</v>
       </c>
-      <c r="B37" s="148"/>
-      <c r="C37" s="148"/>
-      <c r="D37" s="148"/>
-      <c r="E37" s="148"/>
-      <c r="F37" s="148"/>
-      <c r="G37" s="148"/>
+      <c r="B37" s="146"/>
+      <c r="C37" s="146"/>
+      <c r="D37" s="146"/>
+      <c r="E37" s="146"/>
+      <c r="F37" s="146"/>
+      <c r="G37" s="146"/>
       <c r="J37" s="52"/>
     </row>
-    <row r="38" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="38" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="36" t="s">
         <v>53</v>
       </c>
@@ -2967,7 +2964,7 @@
       <c r="M38" s="54"/>
       <c r="N38" s="54"/>
     </row>
-    <row r="39" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="39" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="36" t="s">
         <v>54</v>
       </c>
@@ -2977,45 +2974,45 @@
       <c r="M39" s="54"/>
       <c r="N39" s="54"/>
     </row>
-    <row r="40" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A40" s="148" t="s">
+    <row r="40" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="146" t="s">
         <v>55</v>
       </c>
-      <c r="B40" s="148"/>
-      <c r="C40" s="148"/>
-      <c r="D40" s="148"/>
-      <c r="E40" s="148"/>
-      <c r="F40" s="148"/>
-      <c r="G40" s="148"/>
+      <c r="B40" s="146"/>
+      <c r="C40" s="146"/>
+      <c r="D40" s="146"/>
+      <c r="E40" s="146"/>
+      <c r="F40" s="146"/>
+      <c r="G40" s="146"/>
       <c r="J40" s="52"/>
     </row>
-    <row r="41" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A41" s="166" t="s">
+    <row r="41" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="164" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="166"/>
-      <c r="C41" s="166"/>
-      <c r="D41" s="166"/>
-      <c r="E41" s="166"/>
-      <c r="F41" s="166"/>
-      <c r="G41" s="166"/>
+      <c r="B41" s="164"/>
+      <c r="C41" s="164"/>
+      <c r="D41" s="164"/>
+      <c r="E41" s="164"/>
+      <c r="F41" s="164"/>
+      <c r="G41" s="164"/>
       <c r="M41" s="54"/>
       <c r="N41" s="54"/>
     </row>
-    <row r="42" spans="1:14" s="6" customFormat="1" ht="44.25" customHeight="1">
-      <c r="A42" s="162" t="s">
+    <row r="42" spans="1:14" s="6" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="160" t="s">
         <v>57</v>
       </c>
-      <c r="B42" s="162"/>
-      <c r="C42" s="162"/>
-      <c r="D42" s="162"/>
-      <c r="E42" s="162"/>
-      <c r="F42" s="162"/>
-      <c r="G42" s="162"/>
+      <c r="B42" s="160"/>
+      <c r="C42" s="160"/>
+      <c r="D42" s="160"/>
+      <c r="E42" s="160"/>
+      <c r="F42" s="160"/>
+      <c r="G42" s="160"/>
       <c r="M42" s="54"/>
       <c r="N42" s="54"/>
     </row>
-    <row r="43" spans="1:14" s="4" customFormat="1" ht="7.5" customHeight="1">
+    <row r="43" spans="1:14" s="4" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="35"/>
       <c r="B43" s="35"/>
       <c r="C43" s="35"/>
@@ -3025,32 +3022,32 @@
       <c r="G43" s="35"/>
       <c r="J43" s="52"/>
     </row>
-    <row r="44" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A44" s="148" t="s">
+    <row r="44" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="146" t="s">
         <v>58</v>
       </c>
-      <c r="B44" s="148"/>
-      <c r="C44" s="148"/>
-      <c r="D44" s="148"/>
-      <c r="E44" s="148"/>
-      <c r="F44" s="148"/>
-      <c r="G44" s="148"/>
+      <c r="B44" s="146"/>
+      <c r="C44" s="146"/>
+      <c r="D44" s="146"/>
+      <c r="E44" s="146"/>
+      <c r="F44" s="146"/>
+      <c r="G44" s="146"/>
       <c r="J44" s="52"/>
     </row>
-    <row r="45" spans="1:14" s="6" customFormat="1" ht="58.5" customHeight="1">
-      <c r="A45" s="163" t="s">
+    <row r="45" spans="1:14" s="6" customFormat="1" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="161" t="s">
         <v>59</v>
       </c>
-      <c r="B45" s="164"/>
-      <c r="C45" s="164"/>
-      <c r="D45" s="164"/>
-      <c r="E45" s="164"/>
-      <c r="F45" s="164"/>
-      <c r="G45" s="164"/>
+      <c r="B45" s="162"/>
+      <c r="C45" s="162"/>
+      <c r="D45" s="162"/>
+      <c r="E45" s="162"/>
+      <c r="F45" s="162"/>
+      <c r="G45" s="162"/>
       <c r="M45" s="54"/>
       <c r="N45" s="54"/>
     </row>
-    <row r="46" spans="1:14" s="4" customFormat="1" ht="7.5" customHeight="1">
+    <row r="46" spans="1:14" s="4" customFormat="1" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="35"/>
       <c r="B46" s="35"/>
       <c r="C46" s="35"/>
@@ -3060,32 +3057,32 @@
       <c r="G46" s="35"/>
       <c r="J46" s="52"/>
     </row>
-    <row r="47" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1">
-      <c r="A47" s="148" t="s">
+    <row r="47" spans="1:14" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="146" t="s">
         <v>60</v>
       </c>
-      <c r="B47" s="148"/>
-      <c r="C47" s="148"/>
-      <c r="D47" s="148"/>
-      <c r="E47" s="148"/>
-      <c r="F47" s="148"/>
-      <c r="G47" s="148"/>
+      <c r="B47" s="146"/>
+      <c r="C47" s="146"/>
+      <c r="D47" s="146"/>
+      <c r="E47" s="146"/>
+      <c r="F47" s="146"/>
+      <c r="G47" s="146"/>
       <c r="J47" s="52"/>
     </row>
-    <row r="48" spans="1:14" s="6" customFormat="1" ht="46.5" customHeight="1">
-      <c r="A48" s="165" t="s">
+    <row r="48" spans="1:14" s="6" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="163" t="s">
         <v>61</v>
       </c>
-      <c r="B48" s="165"/>
-      <c r="C48" s="165"/>
-      <c r="D48" s="165"/>
-      <c r="E48" s="165"/>
-      <c r="F48" s="165"/>
-      <c r="G48" s="165"/>
+      <c r="B48" s="163"/>
+      <c r="C48" s="163"/>
+      <c r="D48" s="163"/>
+      <c r="E48" s="163"/>
+      <c r="F48" s="163"/>
+      <c r="G48" s="163"/>
       <c r="M48" s="54"/>
       <c r="N48" s="54"/>
     </row>
-    <row r="49" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="49" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="36"/>
       <c r="C49" s="36"/>
       <c r="D49" s="36"/>
@@ -3093,20 +3090,20 @@
       <c r="M49" s="54"/>
       <c r="N49" s="54"/>
     </row>
-    <row r="50" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
-      <c r="A50" s="148" t="s">
+    <row r="50" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="146" t="s">
         <v>62</v>
       </c>
-      <c r="B50" s="148"/>
-      <c r="C50" s="148"/>
-      <c r="D50" s="148"/>
-      <c r="E50" s="148"/>
-      <c r="F50" s="148"/>
-      <c r="G50" s="148"/>
+      <c r="B50" s="146"/>
+      <c r="C50" s="146"/>
+      <c r="D50" s="146"/>
+      <c r="E50" s="146"/>
+      <c r="F50" s="146"/>
+      <c r="G50" s="146"/>
       <c r="M50" s="54"/>
       <c r="N50" s="54"/>
     </row>
-    <row r="51" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="51" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="39" t="s">
         <v>63</v>
       </c>
@@ -3121,7 +3118,7 @@
       <c r="M51" s="54"/>
       <c r="N51" s="54"/>
     </row>
-    <row r="52" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1">
+    <row r="52" spans="1:14" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="40" t="str">
         <f>B4</f>
         <v>CHONGQING ALUSTARS INTERNATIONAL CO.,LTD.</v>
@@ -3137,7 +3134,7 @@
       <c r="M52" s="54"/>
       <c r="N52" s="54"/>
     </row>
-    <row r="53" spans="1:14">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="36" t="s">
         <v>65</v>
       </c>
@@ -3148,7 +3145,7 @@
       </c>
       <c r="G53" s="44"/>
     </row>
-    <row r="54" spans="1:14">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="36" t="s">
         <v>66</v>
       </c>

</xml_diff>